<commit_message>
cambios pre-reunion, pruebas unitarias HU-17,HU-18
</commit_message>
<xml_diff>
--- a/data/datos_reales/xlsx/DatosReales_CICES_Personal.xlsx
+++ b/data/datos_reales/xlsx/DatosReales_CICES_Personal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angie\IdeaProjects\cices-system\data\datos_reales\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{235B5626-1A35-4AA9-98E9-6C025DC83F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D27D25A-6132-4F6E-8E01-C82FA1137FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="USUARIO" sheetId="1" r:id="rId1"/>
@@ -47,646 +47,646 @@
     <t>analaura.solanolopez@ucr.ac.cr</t>
   </si>
   <si>
+    <t>derby.munoz@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>jeanneth.cerdas@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>yamileth.chacon@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>cinthyacordoba@gmail.com</t>
+  </si>
+  <si>
+    <t>ingrid.gomez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>karla.martorell@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>jose.moncada@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>eiliana.montero@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>benjamin.reyesfernandez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>mariela.rodriguezvalerio@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>maria.saenzmadrigal@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>sedali.solis@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>beatriz.villalobos@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>maria.martinezhernandez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>jerik.andradeespinales@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>claudia.arauz@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>agustin.arguedas@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>jaimealonso.caravaca@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>priscilla.carmiol@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>cristobal.chingalvarez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>sunny.gonzalez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>sophia.gonzalez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>viriam.leiva@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>dilana.lopezborbon@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>laura.lopeznavarro@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>daniel.martinezesquivel@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>maritza.mata@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ana.quezadaugalde@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>noe.ramirez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>katherine.salazarrojas@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>hanna.sanabriabarahona@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>vivian.vilchez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>katherine.soliscordero@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ejemplo1@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ejemplo2@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ejemplo3@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ejemplo4@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ejemplo5@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ejemplo6@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>natalie.padilla@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>jimena.chaconalvarez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ericka.murillo@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>karolcristina.rojas@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>jaime.fornaguera@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>anacecilia.zuniga@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>mariajose.cordero@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>carlose.mora@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>jennifer.gutierrez@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>ID_EMPLEADO</t>
+  </si>
+  <si>
+    <t>NOMBRE_COMPLETO</t>
+  </si>
+  <si>
+    <t>IDENTIFICACION</t>
+  </si>
+  <si>
+    <t>ID_CODIGO_TIPO_ID</t>
+  </si>
+  <si>
+    <t>PAIS</t>
+  </si>
+  <si>
+    <t>CORREO</t>
+  </si>
+  <si>
+    <t>NUMERO_TELEFONO</t>
+  </si>
+  <si>
+    <t>ID_CODIGO_TIPO_GRADO_ACADEMICO</t>
+  </si>
+  <si>
+    <t>Ana Laura Solano López</t>
+  </si>
+  <si>
+    <t>CR</t>
+  </si>
+  <si>
+    <t>Derby Muñoz Rojas</t>
+  </si>
+  <si>
+    <t>Jeannette Cerdas Núñez</t>
+  </si>
+  <si>
+    <t>8339-3707</t>
+  </si>
+  <si>
+    <t>Yamileth Chacón Araya</t>
+  </si>
+  <si>
+    <t>Cinthya Córdoba López</t>
+  </si>
+  <si>
+    <t>8843-3888</t>
+  </si>
+  <si>
+    <t>Ingrid Gómez-Duarte</t>
+  </si>
+  <si>
+    <t>Karla Martorell Esquivel</t>
+  </si>
+  <si>
+    <t>Jose Moncada Jiménez</t>
+  </si>
+  <si>
+    <t>Eiliana Montero Rojas</t>
+  </si>
+  <si>
+    <t>8839-4472</t>
+  </si>
+  <si>
+    <t>Benjamín Reyes Fernández</t>
+  </si>
+  <si>
+    <t>2511-6978</t>
+  </si>
+  <si>
+    <t>Mariela Francine Rodríguez Valerio</t>
+  </si>
+  <si>
+    <t>María Sáenz Madrigal</t>
+  </si>
+  <si>
+    <t>Sedali Solís Agüero</t>
+  </si>
+  <si>
+    <t>Beatriz Villalobos Núñez</t>
+  </si>
+  <si>
+    <t>María del Rocío Martínez Hernández</t>
+  </si>
+  <si>
+    <t>8529-8000</t>
+  </si>
+  <si>
+    <t>Jerik Antonio Andrade Espinales</t>
+  </si>
+  <si>
+    <t>NI</t>
+  </si>
+  <si>
+    <t>Claudia Patricia Arauz Mendoza</t>
+  </si>
+  <si>
+    <t>José Agustín Arguedas Quesada</t>
+  </si>
+  <si>
+    <t>Jaime Alonso Caravaca Morera</t>
+  </si>
+  <si>
+    <t>Priscila Carmiol Rodríguez</t>
+  </si>
+  <si>
+    <t>Cristóbal Ching Álvarez</t>
+  </si>
+  <si>
+    <t>8374-3444</t>
+  </si>
+  <si>
+    <t>Sunny González Serrano</t>
+  </si>
+  <si>
+    <t>Sophía Mariela González Zúñiga</t>
+  </si>
+  <si>
+    <t>Viriam Leiva Díaz</t>
+  </si>
+  <si>
+    <t>Dilana López Borbón</t>
+  </si>
+  <si>
+    <t>Laura Daniela López Navarro</t>
+  </si>
+  <si>
+    <t>Daniel Martínez Esquivel</t>
+  </si>
+  <si>
+    <t>Maritza Mata Barahona</t>
+  </si>
+  <si>
+    <t>Ana María Quezada Ugalde</t>
+  </si>
+  <si>
+    <t>Noé Alberto Ramírez Elizondo</t>
+  </si>
+  <si>
+    <t>Katherine Paola Salazar Rojas</t>
+  </si>
+  <si>
+    <t>Hanna Sanabria Barahona</t>
+  </si>
+  <si>
+    <t>Vivian Vilchez Barboza</t>
+  </si>
+  <si>
+    <t>Katherine Solís Cordero</t>
+  </si>
+  <si>
+    <t>Jorge Vinicio Fallas Herrera</t>
+  </si>
+  <si>
+    <t>Adriana María Guerrero Ramírez</t>
+  </si>
+  <si>
+    <t>Yerlin María Quesada Rodríguez</t>
+  </si>
+  <si>
+    <t>Patsy Marcela Quesada Carballo</t>
+  </si>
+  <si>
+    <t>Yerlin Ramírez Chavarría</t>
+  </si>
+  <si>
+    <t>María Carolina RodrígueAz Bonilla</t>
+  </si>
+  <si>
+    <t>Natalie Padilla Ureña</t>
+  </si>
+  <si>
+    <t>Jimena Chacón Alvarez</t>
+  </si>
+  <si>
+    <t>Ericka Carolina Murillo Rodríguez</t>
+  </si>
+  <si>
+    <t>Karol Cristina Rojas Araya</t>
+  </si>
+  <si>
+    <t>Jaime Fornaguera Trías</t>
+  </si>
+  <si>
+    <t>Ana Cecilia Zúñiga González</t>
+  </si>
+  <si>
+    <t>María José Cordero López</t>
+  </si>
+  <si>
+    <t>Carlos Eduardo Mora Campos</t>
+  </si>
+  <si>
+    <t>Jennifer Leticia Gutierrez Rivera</t>
+  </si>
+  <si>
+    <t>ID_ROL</t>
+  </si>
+  <si>
+    <t>ID_ROL_USUARIO</t>
+  </si>
+  <si>
+    <t>ID_INVESTIGADOR</t>
+  </si>
+  <si>
+    <t>ID_UNIDAD_ACADEMICA</t>
+  </si>
+  <si>
+    <t>ID_INSTITUCION_ORIGEN</t>
+  </si>
+  <si>
+    <t>TEMA_INTERES</t>
+  </si>
+  <si>
+    <t>Salud y bienestar</t>
+  </si>
+  <si>
+    <t>Factores psicosociales y conductas de riesgo en jóvenes</t>
+  </si>
+  <si>
+    <t>Interacción pedagógica en educación inicial</t>
+  </si>
+  <si>
+    <t>Políticas públicas, salud y evaluación de servicios</t>
+  </si>
+  <si>
+    <t>Salud pública, epidemiología y promoción de la salud</t>
+  </si>
+  <si>
+    <t>Fisiología del ejercicio y genética deportiva</t>
+  </si>
+  <si>
+    <t>Psicometría, medición psicológica y educativa, desarrollo psicológico</t>
+  </si>
+  <si>
+    <t>Investigación en enfermería, cuidado y salud</t>
+  </si>
+  <si>
+    <t>Salud pública, simulación clínica, investigación en enfermería</t>
+  </si>
+  <si>
+    <t>Salud colectiva, justicia social e inequidades en salud</t>
+  </si>
+  <si>
+    <t>Burnout en cuidadores de personas adultas mayores</t>
+  </si>
+  <si>
+    <t>Enfermería pediátrica en niñez y adolescencia</t>
+  </si>
+  <si>
+    <t>Duelo, continuidad de vínculos y conductas suicidas</t>
+  </si>
+  <si>
+    <t>Farmacodependencia y neuropsicología</t>
+  </si>
+  <si>
+    <t>Desarrollo infantil, adaptación familiar y salud mental infantil</t>
+  </si>
+  <si>
+    <t>Enfermería en salud colectiva</t>
+  </si>
+  <si>
+    <t>ID_TITULO</t>
+  </si>
+  <si>
+    <t>NOMBRE_TITULO</t>
+  </si>
+  <si>
+    <t>ID_CODIGO_TIPO_NIVEL_TITULO</t>
+  </si>
+  <si>
+    <t>ID_ENTIDAD</t>
+  </si>
+  <si>
+    <t>FECHA_EMISION</t>
+  </si>
+  <si>
+    <t>PhD en Enfermería</t>
+  </si>
+  <si>
+    <t>Maestría en Informática en Salud</t>
+  </si>
+  <si>
+    <t>Licenciatura en Enfermería</t>
+  </si>
+  <si>
+    <t>Doctorado en Filosofía en Enfermería</t>
+  </si>
+  <si>
+    <t>Maestría Académica en Ciencias del Movimiento Humano</t>
+  </si>
+  <si>
+    <t>Maestría en Planificación Curricular</t>
+  </si>
+  <si>
+    <t>Licenciatura en Educación Preescolar</t>
+  </si>
+  <si>
+    <t>Máster en Psicología Clínica y de la Salud</t>
+  </si>
+  <si>
+    <t>Máster en Administración de Servicios de Salud Sostenible</t>
+  </si>
+  <si>
+    <t>Doctorado en Epidemiología y Salud Pública</t>
+  </si>
+  <si>
+    <t>Maestría en Epidemiología y Salud Pública</t>
+  </si>
+  <si>
+    <t>Licenciatura en Medicina y Cirugía</t>
+  </si>
+  <si>
+    <t>Ph.D. en Investigación Educativa (Evaluación y Medición)</t>
+  </si>
+  <si>
+    <t>M.Sc. en Investigación Educativa (Evaluación y Medición)</t>
+  </si>
+  <si>
+    <t>Bachillerato en Estadística</t>
+  </si>
+  <si>
+    <t>Doctorado en Psicología</t>
+  </si>
+  <si>
+    <t>Magister en Psicología Clínica y de la Salud</t>
+  </si>
+  <si>
+    <t>Licenciatura en Psicología</t>
+  </si>
+  <si>
+    <t>Bachillerato en Psicología</t>
+  </si>
+  <si>
+    <t>Maestría Profesional en Salud Pública con énfasis en Gerencia de la Salud</t>
+  </si>
+  <si>
+    <t>Doctorado en Salud Colectiva con énfasis en Justicia Social</t>
+  </si>
+  <si>
+    <t>Maestría en Salud Colectiva</t>
+  </si>
+  <si>
+    <t>Magister en Ciencias de la Enfermería (Salud Laboral)</t>
+  </si>
+  <si>
+    <t>Diplomado en Teología</t>
+  </si>
+  <si>
+    <t>Diplomado en Administración en Salud Ocupacional</t>
+  </si>
+  <si>
+    <t>Maestría Académica en Docencia Universitaria</t>
+  </si>
+  <si>
+    <t>Maestría Profesional en Gestión del Riesgo de Desastres y Atención de Emergencias</t>
+  </si>
+  <si>
+    <t>Maestría Profesional en Enfermería Pediátrica con énfasis en Niñez y Adolescencia</t>
+  </si>
+  <si>
+    <t>Diplomado en Administración de Servicios de Salud Sostenible</t>
+  </si>
+  <si>
+    <t>Maestría Profesional en Enfermería de Salud Mental</t>
+  </si>
+  <si>
+    <t>Doctorado en Ciencias Médicas y Farmacéuticas, Desarrollo y Calidad de Vida</t>
+  </si>
+  <si>
+    <t>Bachillerato y Licenciatura en Psicología</t>
+  </si>
+  <si>
+    <t>Maestría Académica en Farmacodependencia</t>
+  </si>
+  <si>
+    <t>Diplomado en Neuroanatomía Funcional con orientación Clínica</t>
+  </si>
+  <si>
+    <t>Maestría en Enfermería Pediátrica con énfasis en Niñez y Adolescencia</t>
+  </si>
+  <si>
+    <t>Bachiller en Educación Media</t>
+  </si>
+  <si>
+    <t>Doctorado en Ciencias – Área de concentración Enfermería en Salud Colectiva</t>
+  </si>
+  <si>
+    <t>ID_CERTIFICACION</t>
+  </si>
+  <si>
+    <t>NOMBRE_CERTIFICACION</t>
+  </si>
+  <si>
+    <t>ID_CODIGO_TIPO_CERTIFICACION</t>
+  </si>
+  <si>
+    <t>FECHA_EXPIRACION</t>
+  </si>
+  <si>
+    <t>ID_CODIGO_TIPO_ESTADO</t>
+  </si>
+  <si>
+    <t>Investigadora observacional e intervencional</t>
+  </si>
+  <si>
+    <t>Enfermero registrado #E-6748</t>
+  </si>
+  <si>
+    <t>Investigador intervencional acreditado (#153-2016 / #2507-2019)</t>
+  </si>
+  <si>
+    <t>Especialista en Monitoreo y Evaluación para la Gestión de Políticas y Programas de VIH y sida</t>
+  </si>
+  <si>
+    <t>Posgrado en Evaluación de Efectividad en Salud Pública: Promoción de la Salud y Atención Primaria</t>
+  </si>
+  <si>
+    <t>Posgrado en Evaluación de Resultados e Impactos de Organizaciones y Programas Públicos</t>
+  </si>
+  <si>
+    <t>Posgrado en Gestión Local de Salud</t>
+  </si>
+  <si>
+    <t>Certificación como Investigadora Secundaria</t>
+  </si>
+  <si>
+    <t>Soporte Vital Cardiovascular Avanzado</t>
+  </si>
+  <si>
+    <t>Buenas prácticas clínicas</t>
+  </si>
+  <si>
+    <t>Instructor en Soporte Vital Básico</t>
+  </si>
+  <si>
+    <t>Autorización como Investigador Principal para estudios observacionales</t>
+  </si>
+  <si>
+    <t>Soporte Cardíaco Avanzado Pediátrico</t>
+  </si>
+  <si>
+    <t>Instructor en Simulación Clínica</t>
+  </si>
+  <si>
+    <t>Instructor Internacional Asociación Americana del Corazón (AHA)</t>
+  </si>
+  <si>
+    <t>Instructor Internacional en Simulación Clínica</t>
+  </si>
+  <si>
+    <t>Proveedor Soporte Vital Pre-hospitalario en Trauma (PHTLS)</t>
+  </si>
+  <si>
+    <t>Medicina Táctica y Trauma Avanzado (Fénix III)</t>
+  </si>
+  <si>
+    <t>Investigador Observacional Principal</t>
+  </si>
+  <si>
+    <t>Certificado de Graduación de Honor (Promedio 9.19)</t>
+  </si>
+  <si>
+    <t>Curso Soporte Cardiovascular Básico</t>
+  </si>
+  <si>
+    <t>II Curso Latinoamericano de Instructores en Simulación Clínica</t>
+  </si>
+  <si>
+    <t>TeamSTEPPS Essentials Course</t>
+  </si>
+  <si>
+    <t>Consejerías en alcohol y otras drogas</t>
+  </si>
+  <si>
+    <t>Intervenciones innovadoras E-Health en la investigación</t>
+  </si>
+  <si>
+    <t>Curso Buenas Prácticas Clínicas y Bioética</t>
+  </si>
+  <si>
+    <t>Neuropsicología cognitiva</t>
+  </si>
+  <si>
+    <t>Intercambio académico en Clinical Nursing y Pediatric Nursing Care</t>
+  </si>
+  <si>
+    <t>Pasantía doctoral</t>
+  </si>
+  <si>
+    <t>Pasantía de maestría</t>
+  </si>
+  <si>
+    <t>Actualización en el manejo de desechos sólidos hospitalarios y técnicas aséptica médico quirúrgica</t>
+  </si>
+  <si>
     <t>$2a$10$kWDYd0ioPAF98lxQHAxGaewL3jBNgGqTFwn95532pPwCAKETwTKae</t>
-  </si>
-  <si>
-    <t>derby.munoz@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>jeanneth.cerdas@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>yamileth.chacon@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>cinthyacordoba@gmail.com</t>
-  </si>
-  <si>
-    <t>ingrid.gomez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>karla.martorell@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>jose.moncada@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>eiliana.montero@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>benjamin.reyesfernandez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>mariela.rodriguezvalerio@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>maria.saenzmadrigal@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>sedali.solis@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>beatriz.villalobos@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>maria.martinezhernandez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>jerik.andradeespinales@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>claudia.arauz@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>agustin.arguedas@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>jaimealonso.caravaca@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>priscilla.carmiol@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>cristobal.chingalvarez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>sunny.gonzalez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>sophia.gonzalez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>viriam.leiva@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>dilana.lopezborbon@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>laura.lopeznavarro@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>daniel.martinezesquivel@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>maritza.mata@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ana.quezadaugalde@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>noe.ramirez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>katherine.salazarrojas@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>hanna.sanabriabarahona@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>vivian.vilchez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>katherine.soliscordero@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ejemplo1@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ejemplo2@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ejemplo3@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ejemplo4@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ejemplo5@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ejemplo6@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>natalie.padilla@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>jimena.chaconalvarez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ericka.murillo@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>karolcristina.rojas@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>jaime.fornaguera@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>anacecilia.zuniga@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>mariajose.cordero@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>carlose.mora@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>jennifer.gutierrez@ucr.ac.cr</t>
-  </si>
-  <si>
-    <t>ID_EMPLEADO</t>
-  </si>
-  <si>
-    <t>NOMBRE_COMPLETO</t>
-  </si>
-  <si>
-    <t>IDENTIFICACION</t>
-  </si>
-  <si>
-    <t>ID_CODIGO_TIPO_ID</t>
-  </si>
-  <si>
-    <t>PAIS</t>
-  </si>
-  <si>
-    <t>CORREO</t>
-  </si>
-  <si>
-    <t>NUMERO_TELEFONO</t>
-  </si>
-  <si>
-    <t>ID_CODIGO_TIPO_GRADO_ACADEMICO</t>
-  </si>
-  <si>
-    <t>Ana Laura Solano López</t>
-  </si>
-  <si>
-    <t>CR</t>
-  </si>
-  <si>
-    <t>Derby Muñoz Rojas</t>
-  </si>
-  <si>
-    <t>Jeannette Cerdas Núñez</t>
-  </si>
-  <si>
-    <t>8339-3707</t>
-  </si>
-  <si>
-    <t>Yamileth Chacón Araya</t>
-  </si>
-  <si>
-    <t>Cinthya Córdoba López</t>
-  </si>
-  <si>
-    <t>8843-3888</t>
-  </si>
-  <si>
-    <t>Ingrid Gómez-Duarte</t>
-  </si>
-  <si>
-    <t>Karla Martorell Esquivel</t>
-  </si>
-  <si>
-    <t>Jose Moncada Jiménez</t>
-  </si>
-  <si>
-    <t>Eiliana Montero Rojas</t>
-  </si>
-  <si>
-    <t>8839-4472</t>
-  </si>
-  <si>
-    <t>Benjamín Reyes Fernández</t>
-  </si>
-  <si>
-    <t>2511-6978</t>
-  </si>
-  <si>
-    <t>Mariela Francine Rodríguez Valerio</t>
-  </si>
-  <si>
-    <t>María Sáenz Madrigal</t>
-  </si>
-  <si>
-    <t>Sedali Solís Agüero</t>
-  </si>
-  <si>
-    <t>Beatriz Villalobos Núñez</t>
-  </si>
-  <si>
-    <t>María del Rocío Martínez Hernández</t>
-  </si>
-  <si>
-    <t>8529-8000</t>
-  </si>
-  <si>
-    <t>Jerik Antonio Andrade Espinales</t>
-  </si>
-  <si>
-    <t>NI</t>
-  </si>
-  <si>
-    <t>Claudia Patricia Arauz Mendoza</t>
-  </si>
-  <si>
-    <t>José Agustín Arguedas Quesada</t>
-  </si>
-  <si>
-    <t>Jaime Alonso Caravaca Morera</t>
-  </si>
-  <si>
-    <t>Priscila Carmiol Rodríguez</t>
-  </si>
-  <si>
-    <t>Cristóbal Ching Álvarez</t>
-  </si>
-  <si>
-    <t>8374-3444</t>
-  </si>
-  <si>
-    <t>Sunny González Serrano</t>
-  </si>
-  <si>
-    <t>Sophía Mariela González Zúñiga</t>
-  </si>
-  <si>
-    <t>Viriam Leiva Díaz</t>
-  </si>
-  <si>
-    <t>Dilana López Borbón</t>
-  </si>
-  <si>
-    <t>Laura Daniela López Navarro</t>
-  </si>
-  <si>
-    <t>Daniel Martínez Esquivel</t>
-  </si>
-  <si>
-    <t>Maritza Mata Barahona</t>
-  </si>
-  <si>
-    <t>Ana María Quezada Ugalde</t>
-  </si>
-  <si>
-    <t>Noé Alberto Ramírez Elizondo</t>
-  </si>
-  <si>
-    <t>Katherine Paola Salazar Rojas</t>
-  </si>
-  <si>
-    <t>Hanna Sanabria Barahona</t>
-  </si>
-  <si>
-    <t>Vivian Vilchez Barboza</t>
-  </si>
-  <si>
-    <t>Katherine Solís Cordero</t>
-  </si>
-  <si>
-    <t>Jorge Vinicio Fallas Herrera</t>
-  </si>
-  <si>
-    <t>Adriana María Guerrero Ramírez</t>
-  </si>
-  <si>
-    <t>Yerlin María Quesada Rodríguez</t>
-  </si>
-  <si>
-    <t>Patsy Marcela Quesada Carballo</t>
-  </si>
-  <si>
-    <t>Yerlin Ramírez Chavarría</t>
-  </si>
-  <si>
-    <t>María Carolina RodrígueAz Bonilla</t>
-  </si>
-  <si>
-    <t>Natalie Padilla Ureña</t>
-  </si>
-  <si>
-    <t>Jimena Chacón Alvarez</t>
-  </si>
-  <si>
-    <t>Ericka Carolina Murillo Rodríguez</t>
-  </si>
-  <si>
-    <t>Karol Cristina Rojas Araya</t>
-  </si>
-  <si>
-    <t>Jaime Fornaguera Trías</t>
-  </si>
-  <si>
-    <t>Ana Cecilia Zúñiga González</t>
-  </si>
-  <si>
-    <t>María José Cordero López</t>
-  </si>
-  <si>
-    <t>Carlos Eduardo Mora Campos</t>
-  </si>
-  <si>
-    <t>Jennifer Leticia Gutierrez Rivera</t>
-  </si>
-  <si>
-    <t>ID_ROL</t>
-  </si>
-  <si>
-    <t>ID_ROL_USUARIO</t>
-  </si>
-  <si>
-    <t>ID_INVESTIGADOR</t>
-  </si>
-  <si>
-    <t>ID_UNIDAD_ACADEMICA</t>
-  </si>
-  <si>
-    <t>ID_INSTITUCION_ORIGEN</t>
-  </si>
-  <si>
-    <t>TEMA_INTERES</t>
-  </si>
-  <si>
-    <t>Salud y bienestar</t>
-  </si>
-  <si>
-    <t>Factores psicosociales y conductas de riesgo en jóvenes</t>
-  </si>
-  <si>
-    <t>Interacción pedagógica en educación inicial</t>
-  </si>
-  <si>
-    <t>Políticas públicas, salud y evaluación de servicios</t>
-  </si>
-  <si>
-    <t>Salud pública, epidemiología y promoción de la salud</t>
-  </si>
-  <si>
-    <t>Fisiología del ejercicio y genética deportiva</t>
-  </si>
-  <si>
-    <t>Psicometría, medición psicológica y educativa, desarrollo psicológico</t>
-  </si>
-  <si>
-    <t>Investigación en enfermería, cuidado y salud</t>
-  </si>
-  <si>
-    <t>Salud pública, simulación clínica, investigación en enfermería</t>
-  </si>
-  <si>
-    <t>Salud colectiva, justicia social e inequidades en salud</t>
-  </si>
-  <si>
-    <t>Burnout en cuidadores de personas adultas mayores</t>
-  </si>
-  <si>
-    <t>Enfermería pediátrica en niñez y adolescencia</t>
-  </si>
-  <si>
-    <t>Duelo, continuidad de vínculos y conductas suicidas</t>
-  </si>
-  <si>
-    <t>Farmacodependencia y neuropsicología</t>
-  </si>
-  <si>
-    <t>Desarrollo infantil, adaptación familiar y salud mental infantil</t>
-  </si>
-  <si>
-    <t>Enfermería en salud colectiva</t>
-  </si>
-  <si>
-    <t>ID_TITULO</t>
-  </si>
-  <si>
-    <t>NOMBRE_TITULO</t>
-  </si>
-  <si>
-    <t>ID_CODIGO_TIPO_NIVEL_TITULO</t>
-  </si>
-  <si>
-    <t>ID_ENTIDAD</t>
-  </si>
-  <si>
-    <t>FECHA_EMISION</t>
-  </si>
-  <si>
-    <t>PhD en Enfermería</t>
-  </si>
-  <si>
-    <t>Maestría en Informática en Salud</t>
-  </si>
-  <si>
-    <t>Licenciatura en Enfermería</t>
-  </si>
-  <si>
-    <t>Doctorado en Filosofía en Enfermería</t>
-  </si>
-  <si>
-    <t>Maestría Académica en Ciencias del Movimiento Humano</t>
-  </si>
-  <si>
-    <t>Maestría en Planificación Curricular</t>
-  </si>
-  <si>
-    <t>Licenciatura en Educación Preescolar</t>
-  </si>
-  <si>
-    <t>Máster en Psicología Clínica y de la Salud</t>
-  </si>
-  <si>
-    <t>Máster en Administración de Servicios de Salud Sostenible</t>
-  </si>
-  <si>
-    <t>Doctorado en Epidemiología y Salud Pública</t>
-  </si>
-  <si>
-    <t>Maestría en Epidemiología y Salud Pública</t>
-  </si>
-  <si>
-    <t>Licenciatura en Medicina y Cirugía</t>
-  </si>
-  <si>
-    <t>Ph.D. en Investigación Educativa (Evaluación y Medición)</t>
-  </si>
-  <si>
-    <t>M.Sc. en Investigación Educativa (Evaluación y Medición)</t>
-  </si>
-  <si>
-    <t>Bachillerato en Estadística</t>
-  </si>
-  <si>
-    <t>Doctorado en Psicología</t>
-  </si>
-  <si>
-    <t>Magister en Psicología Clínica y de la Salud</t>
-  </si>
-  <si>
-    <t>Licenciatura en Psicología</t>
-  </si>
-  <si>
-    <t>Bachillerato en Psicología</t>
-  </si>
-  <si>
-    <t>Maestría Profesional en Salud Pública con énfasis en Gerencia de la Salud</t>
-  </si>
-  <si>
-    <t>Doctorado en Salud Colectiva con énfasis en Justicia Social</t>
-  </si>
-  <si>
-    <t>Maestría en Salud Colectiva</t>
-  </si>
-  <si>
-    <t>Magister en Ciencias de la Enfermería (Salud Laboral)</t>
-  </si>
-  <si>
-    <t>Diplomado en Teología</t>
-  </si>
-  <si>
-    <t>Diplomado en Administración en Salud Ocupacional</t>
-  </si>
-  <si>
-    <t>Maestría Académica en Docencia Universitaria</t>
-  </si>
-  <si>
-    <t>Maestría Profesional en Gestión del Riesgo de Desastres y Atención de Emergencias</t>
-  </si>
-  <si>
-    <t>Maestría Profesional en Enfermería Pediátrica con énfasis en Niñez y Adolescencia</t>
-  </si>
-  <si>
-    <t>Diplomado en Administración de Servicios de Salud Sostenible</t>
-  </si>
-  <si>
-    <t>Maestría Profesional en Enfermería de Salud Mental</t>
-  </si>
-  <si>
-    <t>Doctorado en Ciencias Médicas y Farmacéuticas, Desarrollo y Calidad de Vida</t>
-  </si>
-  <si>
-    <t>Bachillerato y Licenciatura en Psicología</t>
-  </si>
-  <si>
-    <t>Maestría Académica en Farmacodependencia</t>
-  </si>
-  <si>
-    <t>Diplomado en Neuroanatomía Funcional con orientación Clínica</t>
-  </si>
-  <si>
-    <t>Maestría en Enfermería Pediátrica con énfasis en Niñez y Adolescencia</t>
-  </si>
-  <si>
-    <t>Bachiller en Educación Media</t>
-  </si>
-  <si>
-    <t>Doctorado en Ciencias – Área de concentración Enfermería en Salud Colectiva</t>
-  </si>
-  <si>
-    <t>ID_CERTIFICACION</t>
-  </si>
-  <si>
-    <t>NOMBRE_CERTIFICACION</t>
-  </si>
-  <si>
-    <t>ID_CODIGO_TIPO_CERTIFICACION</t>
-  </si>
-  <si>
-    <t>FECHA_EXPIRACION</t>
-  </si>
-  <si>
-    <t>ID_CODIGO_TIPO_ESTADO</t>
-  </si>
-  <si>
-    <t>Investigadora observacional e intervencional</t>
-  </si>
-  <si>
-    <t>Enfermero registrado #E-6748</t>
-  </si>
-  <si>
-    <t>Investigador intervencional acreditado (#153-2016 / #2507-2019)</t>
-  </si>
-  <si>
-    <t>Especialista en Monitoreo y Evaluación para la Gestión de Políticas y Programas de VIH y sida</t>
-  </si>
-  <si>
-    <t>Posgrado en Evaluación de Efectividad en Salud Pública: Promoción de la Salud y Atención Primaria</t>
-  </si>
-  <si>
-    <t>Posgrado en Evaluación de Resultados e Impactos de Organizaciones y Programas Públicos</t>
-  </si>
-  <si>
-    <t>Posgrado en Gestión Local de Salud</t>
-  </si>
-  <si>
-    <t>Certificación como Investigadora Secundaria</t>
-  </si>
-  <si>
-    <t>Soporte Vital Cardiovascular Avanzado</t>
-  </si>
-  <si>
-    <t>Buenas prácticas clínicas</t>
-  </si>
-  <si>
-    <t>Instructor en Soporte Vital Básico</t>
-  </si>
-  <si>
-    <t>Autorización como Investigador Principal para estudios observacionales</t>
-  </si>
-  <si>
-    <t>Soporte Cardíaco Avanzado Pediátrico</t>
-  </si>
-  <si>
-    <t>Instructor en Simulación Clínica</t>
-  </si>
-  <si>
-    <t>Instructor Internacional Asociación Americana del Corazón (AHA)</t>
-  </si>
-  <si>
-    <t>Instructor Internacional en Simulación Clínica</t>
-  </si>
-  <si>
-    <t>Proveedor Soporte Vital Pre-hospitalario en Trauma (PHTLS)</t>
-  </si>
-  <si>
-    <t>Medicina Táctica y Trauma Avanzado (Fénix III)</t>
-  </si>
-  <si>
-    <t>Investigador Observacional Principal</t>
-  </si>
-  <si>
-    <t>Certificado de Graduación de Honor (Promedio 9.19)</t>
-  </si>
-  <si>
-    <t>Curso Soporte Cardiovascular Básico</t>
-  </si>
-  <si>
-    <t>II Curso Latinoamericano de Instructores en Simulación Clínica</t>
-  </si>
-  <si>
-    <t>TeamSTEPPS Essentials Course</t>
-  </si>
-  <si>
-    <t>Consejerías en alcohol y otras drogas</t>
-  </si>
-  <si>
-    <t>Intervenciones innovadoras E-Health en la investigación</t>
-  </si>
-  <si>
-    <t>Curso Buenas Prácticas Clínicas y Bioética</t>
-  </si>
-  <si>
-    <t>Neuropsicología cognitiva</t>
-  </si>
-  <si>
-    <t>Intercambio académico en Clinical Nursing y Pediatric Nursing Care</t>
-  </si>
-  <si>
-    <t>Pasantía doctoral</t>
-  </si>
-  <si>
-    <t>Pasantía de maestría</t>
-  </si>
-  <si>
-    <t>Actualización en el manejo de desechos sólidos hospitalarios y técnicas aséptica médico quirúrgica</t>
   </si>
 </sst>
 </file>
@@ -1053,8 +1053,8 @@
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>5</v>
+      <c r="C2" t="s">
+        <v>218</v>
       </c>
       <c r="D2" s="4">
         <v>1</v>
@@ -1065,10 +1065,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="4" t="s">
         <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>218</v>
       </c>
       <c r="D3" s="4">
         <v>1</v>
@@ -1079,10 +1079,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>218</v>
       </c>
       <c r="D4" s="4">
         <v>1</v>
@@ -1093,10 +1093,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>218</v>
       </c>
       <c r="D5" s="4">
         <v>1</v>
@@ -1107,10 +1107,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>218</v>
       </c>
       <c r="D6" s="4">
         <v>1</v>
@@ -1121,10 +1121,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>5</v>
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>218</v>
       </c>
       <c r="D7" s="4">
         <v>1</v>
@@ -1135,10 +1135,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>218</v>
       </c>
       <c r="D8" s="4">
         <v>1</v>
@@ -1149,10 +1149,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>5</v>
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>218</v>
       </c>
       <c r="D9" s="4">
         <v>1</v>
@@ -1163,10 +1163,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>5</v>
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>218</v>
       </c>
       <c r="D10" s="4">
         <v>1</v>
@@ -1177,10 +1177,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>5</v>
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>218</v>
       </c>
       <c r="D11" s="4">
         <v>1</v>
@@ -1191,10 +1191,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>5</v>
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>218</v>
       </c>
       <c r="D12" s="4">
         <v>1</v>
@@ -1205,10 +1205,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>5</v>
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>218</v>
       </c>
       <c r="D13" s="4">
         <v>1</v>
@@ -1219,10 +1219,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>5</v>
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>218</v>
       </c>
       <c r="D14" s="4">
         <v>1</v>
@@ -1233,10 +1233,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>5</v>
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>218</v>
       </c>
       <c r="D15" s="4">
         <v>1</v>
@@ -1247,10 +1247,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>5</v>
+        <v>18</v>
+      </c>
+      <c r="C16" t="s">
+        <v>218</v>
       </c>
       <c r="D16" s="4">
         <v>1</v>
@@ -1261,10 +1261,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>5</v>
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>218</v>
       </c>
       <c r="D17" s="4">
         <v>1</v>
@@ -1275,10 +1275,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>5</v>
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>218</v>
       </c>
       <c r="D18" s="4">
         <v>1</v>
@@ -1289,10 +1289,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>5</v>
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>218</v>
       </c>
       <c r="D19" s="4">
         <v>1</v>
@@ -1303,10 +1303,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>5</v>
+        <v>22</v>
+      </c>
+      <c r="C20" t="s">
+        <v>218</v>
       </c>
       <c r="D20" s="4">
         <v>1</v>
@@ -1317,10 +1317,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>5</v>
+        <v>23</v>
+      </c>
+      <c r="C21" t="s">
+        <v>218</v>
       </c>
       <c r="D21" s="4">
         <v>1</v>
@@ -1331,10 +1331,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>5</v>
+        <v>24</v>
+      </c>
+      <c r="C22" t="s">
+        <v>218</v>
       </c>
       <c r="D22" s="4">
         <v>1</v>
@@ -1345,10 +1345,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>5</v>
+        <v>25</v>
+      </c>
+      <c r="C23" t="s">
+        <v>218</v>
       </c>
       <c r="D23" s="4">
         <v>1</v>
@@ -1359,10 +1359,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>5</v>
+        <v>26</v>
+      </c>
+      <c r="C24" t="s">
+        <v>218</v>
       </c>
       <c r="D24" s="4">
         <v>1</v>
@@ -1373,10 +1373,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>5</v>
+        <v>27</v>
+      </c>
+      <c r="C25" t="s">
+        <v>218</v>
       </c>
       <c r="D25" s="4">
         <v>1</v>
@@ -1387,10 +1387,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>5</v>
+        <v>28</v>
+      </c>
+      <c r="C26" t="s">
+        <v>218</v>
       </c>
       <c r="D26" s="4">
         <v>1</v>
@@ -1401,10 +1401,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>5</v>
+        <v>29</v>
+      </c>
+      <c r="C27" t="s">
+        <v>218</v>
       </c>
       <c r="D27" s="4">
         <v>1</v>
@@ -1415,10 +1415,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>5</v>
+        <v>30</v>
+      </c>
+      <c r="C28" t="s">
+        <v>218</v>
       </c>
       <c r="D28" s="4">
         <v>1</v>
@@ -1429,10 +1429,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>5</v>
+        <v>31</v>
+      </c>
+      <c r="C29" t="s">
+        <v>218</v>
       </c>
       <c r="D29" s="4">
         <v>1</v>
@@ -1443,10 +1443,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>5</v>
+        <v>32</v>
+      </c>
+      <c r="C30" t="s">
+        <v>218</v>
       </c>
       <c r="D30" s="4">
         <v>1</v>
@@ -1457,10 +1457,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>5</v>
+        <v>33</v>
+      </c>
+      <c r="C31" t="s">
+        <v>218</v>
       </c>
       <c r="D31" s="4">
         <v>1</v>
@@ -1471,10 +1471,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>5</v>
+        <v>34</v>
+      </c>
+      <c r="C32" t="s">
+        <v>218</v>
       </c>
       <c r="D32" s="4">
         <v>1</v>
@@ -1485,10 +1485,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>5</v>
+        <v>35</v>
+      </c>
+      <c r="C33" t="s">
+        <v>218</v>
       </c>
       <c r="D33" s="4">
         <v>1</v>
@@ -1499,10 +1499,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>5</v>
+        <v>36</v>
+      </c>
+      <c r="C34" t="s">
+        <v>218</v>
       </c>
       <c r="D34" s="4">
         <v>1</v>
@@ -1513,10 +1513,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>5</v>
+        <v>37</v>
+      </c>
+      <c r="C35" t="s">
+        <v>218</v>
       </c>
       <c r="D35" s="4">
         <v>1</v>
@@ -1527,10 +1527,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>5</v>
+        <v>38</v>
+      </c>
+      <c r="C36" t="s">
+        <v>218</v>
       </c>
       <c r="D36" s="5">
         <v>0</v>
@@ -1541,10 +1541,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>5</v>
+        <v>39</v>
+      </c>
+      <c r="C37" t="s">
+        <v>218</v>
       </c>
       <c r="D37" s="5">
         <v>0</v>
@@ -1555,10 +1555,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>5</v>
+        <v>40</v>
+      </c>
+      <c r="C38" t="s">
+        <v>218</v>
       </c>
       <c r="D38" s="5">
         <v>0</v>
@@ -1569,10 +1569,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>5</v>
+        <v>41</v>
+      </c>
+      <c r="C39" t="s">
+        <v>218</v>
       </c>
       <c r="D39" s="5">
         <v>0</v>
@@ -1583,10 +1583,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>5</v>
+        <v>42</v>
+      </c>
+      <c r="C40" t="s">
+        <v>218</v>
       </c>
       <c r="D40" s="5">
         <v>0</v>
@@ -1597,10 +1597,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>5</v>
+        <v>43</v>
+      </c>
+      <c r="C41" t="s">
+        <v>218</v>
       </c>
       <c r="D41" s="5">
         <v>0</v>
@@ -1611,10 +1611,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>5</v>
+        <v>44</v>
+      </c>
+      <c r="C42" t="s">
+        <v>218</v>
       </c>
       <c r="D42" s="4">
         <v>1</v>
@@ -1625,10 +1625,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>5</v>
+        <v>45</v>
+      </c>
+      <c r="C43" t="s">
+        <v>218</v>
       </c>
       <c r="D43" s="4">
         <v>1</v>
@@ -1639,10 +1639,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>5</v>
+        <v>46</v>
+      </c>
+      <c r="C44" t="s">
+        <v>218</v>
       </c>
       <c r="D44" s="4">
         <v>1</v>
@@ -1653,10 +1653,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>5</v>
+        <v>47</v>
+      </c>
+      <c r="C45" t="s">
+        <v>218</v>
       </c>
       <c r="D45" s="4">
         <v>1</v>
@@ -1667,10 +1667,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>5</v>
+        <v>48</v>
+      </c>
+      <c r="C46" t="s">
+        <v>218</v>
       </c>
       <c r="D46" s="4">
         <v>1</v>
@@ -1681,10 +1681,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>5</v>
+        <v>49</v>
+      </c>
+      <c r="C47" t="s">
+        <v>218</v>
       </c>
       <c r="D47" s="4">
         <v>1</v>
@@ -1695,10 +1695,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>5</v>
+        <v>50</v>
+      </c>
+      <c r="C48" t="s">
+        <v>218</v>
       </c>
       <c r="D48" s="4">
         <v>1</v>
@@ -1709,10 +1709,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>5</v>
+        <v>51</v>
+      </c>
+      <c r="C49" t="s">
+        <v>218</v>
       </c>
       <c r="D49" s="4">
         <v>1</v>
@@ -1723,10 +1723,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>5</v>
+        <v>52</v>
+      </c>
+      <c r="C50" t="s">
+        <v>218</v>
       </c>
       <c r="D50" s="4">
         <v>1</v>
@@ -2756,31 +2756,31 @@
   <sheetData>
     <row r="1" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="J1" s="1"/>
     </row>
@@ -2792,7 +2792,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2">
         <v>304050852</v>
@@ -2801,7 +2801,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>4</v>
@@ -2822,7 +2822,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D3" s="2">
         <v>303620532</v>
@@ -2831,10 +2831,10 @@
         <v>1</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H3" s="2">
         <v>25112097</v>
@@ -2852,7 +2852,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D4" s="2">
         <v>303090392</v>
@@ -2861,13 +2861,13 @@
         <v>1</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I4" s="2">
         <v>7</v>
@@ -2881,7 +2881,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D5" s="2">
         <v>105540538</v>
@@ -2890,10 +2890,10 @@
         <v>1</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H5" s="7">
         <v>88881003</v>
@@ -2910,7 +2910,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D6" s="2">
         <v>303910277</v>
@@ -2919,13 +2919,13 @@
         <v>1</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I6" s="2">
         <v>8</v>
@@ -2939,7 +2939,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D7" s="2">
         <v>108660046</v>
@@ -2948,10 +2948,10 @@
         <v>1</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H7" s="7">
         <v>88881007</v>
@@ -2968,7 +2968,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D8" s="2">
         <v>109500525</v>
@@ -2977,10 +2977,10 @@
         <v>1</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H8" s="8"/>
       <c r="I8" s="2">
@@ -2995,7 +2995,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D9" s="2">
         <v>107660515</v>
@@ -3004,10 +3004,10 @@
         <v>1</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H9" s="7"/>
       <c r="I9" s="2">
@@ -3022,7 +3022,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D10" s="2">
         <v>105910052</v>
@@ -3031,13 +3031,13 @@
         <v>1</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I10" s="2">
         <v>8</v>
@@ -3051,7 +3051,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D11" s="2">
         <v>110500964</v>
@@ -3060,13 +3060,13 @@
         <v>1</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I11" s="2">
         <v>8</v>
@@ -3080,7 +3080,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12" s="2">
         <v>402090569</v>
@@ -3089,10 +3089,10 @@
         <v>1</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2">
@@ -3107,7 +3107,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D13" s="2">
         <v>900540537</v>
@@ -3116,10 +3116,10 @@
         <v>1</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2">
@@ -3134,7 +3134,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D14" s="2">
         <v>109770013</v>
@@ -3143,10 +3143,10 @@
         <v>1</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H14" s="2">
         <v>88881006</v>
@@ -3163,7 +3163,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D15" s="2">
         <v>602950778</v>
@@ -3172,10 +3172,10 @@
         <v>1</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2">
@@ -3190,7 +3190,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D16" s="2">
         <v>1305010987</v>
@@ -3199,13 +3199,13 @@
         <v>1</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I16" s="2">
         <v>6</v>
@@ -3219,7 +3219,7 @@
         <v>16</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D17" s="2">
         <v>800930919</v>
@@ -3228,10 +3228,10 @@
         <v>1</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2">
@@ -3246,7 +3246,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D18" s="2">
         <v>800600993</v>
@@ -3255,10 +3255,10 @@
         <v>1</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2">
@@ -3273,7 +3273,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D19" s="2">
         <v>302380612</v>
@@ -3282,10 +3282,10 @@
         <v>1</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2">
@@ -3300,7 +3300,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D20" s="2">
         <v>112750015</v>
@@ -3309,10 +3309,10 @@
         <v>1</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2">
@@ -3327,7 +3327,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D21" s="2">
         <v>112330548</v>
@@ -3336,10 +3336,10 @@
         <v>1</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2">
@@ -3354,7 +3354,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D22" s="2">
         <v>700820462</v>
@@ -3363,13 +3363,13 @@
         <v>1</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I22" s="2">
         <v>7</v>
@@ -3383,7 +3383,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D23" s="2">
         <v>900450769</v>
@@ -3392,10 +3392,10 @@
         <v>1</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2">
@@ -3410,7 +3410,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D24" s="2">
         <v>401960193</v>
@@ -3419,10 +3419,10 @@
         <v>1</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H24" s="2">
         <v>89208622</v>
@@ -3439,7 +3439,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D25" s="2">
         <v>105810637</v>
@@ -3448,10 +3448,10 @@
         <v>1</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2">
@@ -3466,7 +3466,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D26" s="2">
         <v>112730930</v>
@@ -3475,10 +3475,10 @@
         <v>1</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2">
@@ -3493,7 +3493,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D27" s="2">
         <v>110200458</v>
@@ -3502,10 +3502,10 @@
         <v>1</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H27" s="2"/>
       <c r="I27" s="2">
@@ -3520,7 +3520,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D28" s="2">
         <v>112650693</v>
@@ -3529,10 +3529,10 @@
         <v>1</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H28" s="6">
         <v>34666297593</v>
@@ -3549,7 +3549,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D29" s="2">
         <v>302650015</v>
@@ -3558,10 +3558,10 @@
         <v>1</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H29" s="2">
         <v>83605910</v>
@@ -3578,7 +3578,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D30" s="2">
         <v>113310443</v>
@@ -3587,10 +3587,10 @@
         <v>1</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H30" s="2">
         <v>88640859</v>
@@ -3607,7 +3607,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D31" s="2">
         <v>111180671</v>
@@ -3616,10 +3616,10 @@
         <v>1</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H31" s="2"/>
       <c r="I31" s="2">
@@ -3634,7 +3634,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D32" s="2">
         <v>114570318</v>
@@ -3643,10 +3643,10 @@
         <v>1</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2">
@@ -3661,7 +3661,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D33" s="2">
         <v>112430433</v>
@@ -3670,10 +3670,10 @@
         <v>1</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H33" s="2"/>
       <c r="I33" s="2">
@@ -3688,7 +3688,7 @@
         <v>33</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D34" s="2">
         <v>110270978</v>
@@ -3697,10 +3697,10 @@
         <v>1</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H34" s="2">
         <v>88881002</v>
@@ -3717,7 +3717,7 @@
         <v>34</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D35" s="2">
         <v>113410656</v>
@@ -3726,10 +3726,10 @@
         <v>1</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H35" s="2"/>
       <c r="I35" s="2">
@@ -3744,7 +3744,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D36" s="2">
         <v>115790196</v>
@@ -3753,10 +3753,10 @@
         <v>1</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2">
@@ -3771,7 +3771,7 @@
         <v>36</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D37" s="2">
         <v>604480424</v>
@@ -3780,10 +3780,10 @@
         <v>1</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2">
@@ -3798,7 +3798,7 @@
         <v>37</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D38" s="2">
         <v>207720136</v>
@@ -3807,10 +3807,10 @@
         <v>1</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2">
@@ -3825,7 +3825,7 @@
         <v>38</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D39" s="2">
         <v>304990526</v>
@@ -3834,10 +3834,10 @@
         <v>1</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2">
@@ -3852,7 +3852,7 @@
         <v>39</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D40" s="2">
         <v>207650530</v>
@@ -3861,10 +3861,10 @@
         <v>1</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2">
@@ -3879,7 +3879,7 @@
         <v>40</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D41" s="2">
         <v>117240412</v>
@@ -3888,10 +3888,10 @@
         <v>1</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H41" s="2"/>
       <c r="I41" s="2">
@@ -3906,7 +3906,7 @@
         <v>41</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D42" s="2">
         <v>118370957</v>
@@ -3915,10 +3915,10 @@
         <v>1</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H42" s="2">
         <v>87588264</v>
@@ -3935,7 +3935,7 @@
         <v>42</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D43" s="2">
         <v>1208590093</v>
@@ -3944,10 +3944,10 @@
         <v>1</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H43" s="2">
         <v>70435884</v>
@@ -3964,7 +3964,7 @@
         <v>43</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D44" s="2">
         <v>114940605</v>
@@ -3973,10 +3973,10 @@
         <v>1</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H44" s="2">
         <v>87409468</v>
@@ -3993,7 +3993,7 @@
         <v>44</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D45" s="2">
         <v>208880003</v>
@@ -4002,10 +4002,10 @@
         <v>1</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H45" s="2">
         <v>25117003</v>
@@ -4022,7 +4022,7 @@
         <v>45</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D46" s="2">
         <v>105770001</v>
@@ -4031,10 +4031,10 @@
         <v>1</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H46" s="2">
         <v>25117004</v>
@@ -4051,7 +4051,7 @@
         <v>46</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D47" s="2">
         <v>105770002</v>
@@ -4060,10 +4060,10 @@
         <v>1</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H47" s="2">
         <v>25117005</v>
@@ -4080,7 +4080,7 @@
         <v>47</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D48" s="2">
         <v>105770003</v>
@@ -4089,10 +4089,10 @@
         <v>1</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H48" s="2">
         <v>25117006</v>
@@ -4109,7 +4109,7 @@
         <v>48</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D49" s="2">
         <v>105770004</v>
@@ -4118,10 +4118,10 @@
         <v>1</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H49" s="2">
         <v>25117007</v>
@@ -4138,7 +4138,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D50" s="2">
         <v>113410210</v>
@@ -4147,10 +4147,10 @@
         <v>1</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H50" s="2">
         <v>87243161</v>
@@ -5178,13 +5178,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6727,19 +6727,19 @@
   <sheetData>
     <row r="1" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6756,7 +6756,7 @@
         <v>3</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6773,7 +6773,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6790,7 +6790,7 @@
         <v>3</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6822,7 +6822,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6839,7 +6839,7 @@
         <v>3</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6871,7 +6871,7 @@
         <v>3</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6888,7 +6888,7 @@
         <v>3</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6905,7 +6905,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6982,7 +6982,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -6999,7 +6999,7 @@
         <v>3</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7046,7 +7046,7 @@
         <v>3</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7078,7 +7078,7 @@
         <v>3</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7110,7 +7110,7 @@
         <v>3</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7172,7 +7172,7 @@
         <v>3</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7189,7 +7189,7 @@
         <v>3</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7206,7 +7206,7 @@
         <v>3</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7283,7 +7283,7 @@
         <v>3</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -8464,22 +8464,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="F1" s="12" t="s">
         <v>144</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8490,7 +8490,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D2" s="13">
         <v>8</v>
@@ -8510,7 +8510,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D3" s="13">
         <v>7</v>
@@ -8530,7 +8530,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D4" s="13">
         <v>6</v>
@@ -8550,7 +8550,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D5" s="13">
         <v>8</v>
@@ -8570,7 +8570,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D6" s="13">
         <v>7</v>
@@ -8590,7 +8590,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D7" s="13">
         <v>6</v>
@@ -8610,7 +8610,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D8" s="13">
         <v>7</v>
@@ -8630,7 +8630,7 @@
         <v>3</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D9" s="13">
         <v>6</v>
@@ -8650,7 +8650,7 @@
         <v>5</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D10" s="13">
         <v>7</v>
@@ -8670,7 +8670,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D11" s="13">
         <v>7</v>
@@ -8690,7 +8690,7 @@
         <v>6</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D12" s="13">
         <v>8</v>
@@ -8710,7 +8710,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D13" s="13">
         <v>7</v>
@@ -8730,7 +8730,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D14" s="13">
         <v>6</v>
@@ -8750,7 +8750,7 @@
         <v>9</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D15" s="13">
         <v>8</v>
@@ -8770,7 +8770,7 @@
         <v>9</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D16" s="13">
         <v>7</v>
@@ -8790,7 +8790,7 @@
         <v>9</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D17" s="13">
         <v>4</v>
@@ -8810,7 +8810,7 @@
         <v>10</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D18" s="13">
         <v>8</v>
@@ -8830,7 +8830,7 @@
         <v>10</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D19" s="13">
         <v>7</v>
@@ -8850,7 +8850,7 @@
         <v>10</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D20" s="13">
         <v>6</v>
@@ -8870,7 +8870,7 @@
         <v>10</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D21" s="13">
         <v>4</v>
@@ -8890,7 +8890,7 @@
         <v>15</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D22" s="13">
         <v>6</v>
@@ -8910,7 +8910,7 @@
         <v>16</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D23" s="13">
         <v>6</v>
@@ -8930,7 +8930,7 @@
         <v>16</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D24" s="13">
         <v>7</v>
@@ -8950,7 +8950,7 @@
         <v>19</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D25" s="13">
         <v>8</v>
@@ -8970,7 +8970,7 @@
         <v>19</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D26" s="13">
         <v>7</v>
@@ -8990,7 +8990,7 @@
         <v>21</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D27" s="13">
         <v>6</v>
@@ -9010,7 +9010,7 @@
         <v>21</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D28" s="13">
         <v>7</v>
@@ -9030,7 +9030,7 @@
         <v>21</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D29" s="13">
         <v>4</v>
@@ -9050,7 +9050,7 @@
         <v>21</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D30" s="13">
         <v>4</v>
@@ -9070,7 +9070,7 @@
         <v>21</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D31" s="13">
         <v>7</v>
@@ -9090,7 +9090,7 @@
         <v>21</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D32" s="13">
         <v>7</v>
@@ -9110,7 +9110,7 @@
         <v>23</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D33" s="13">
         <v>6</v>
@@ -9130,7 +9130,7 @@
         <v>23</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D34" s="13">
         <v>7</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D35" s="13">
         <v>6</v>
@@ -9170,7 +9170,7 @@
         <v>27</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D36" s="13">
         <v>4</v>
@@ -9190,7 +9190,7 @@
         <v>27</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D37" s="13">
         <v>7</v>
@@ -9210,7 +9210,7 @@
         <v>27</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D38" s="13">
         <v>8</v>
@@ -9230,7 +9230,7 @@
         <v>28</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D39" s="13">
         <v>6</v>
@@ -9250,7 +9250,7 @@
         <v>28</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D40" s="13">
         <v>7</v>
@@ -9270,7 +9270,7 @@
         <v>28</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D41" s="13">
         <v>4</v>
@@ -9290,7 +9290,7 @@
         <v>29</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D42" s="13">
         <v>6</v>
@@ -9310,7 +9310,7 @@
         <v>29</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D43" s="13">
         <v>7</v>
@@ -9330,7 +9330,7 @@
         <v>29</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D44" s="13">
         <v>8</v>
@@ -9350,7 +9350,7 @@
         <v>34</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D45" s="13">
         <v>5</v>
@@ -9370,7 +9370,7 @@
         <v>34</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D46" s="13">
         <v>6</v>
@@ -9390,7 +9390,7 @@
         <v>34</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D47" s="13">
         <v>7</v>
@@ -9410,7 +9410,7 @@
         <v>34</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D48" s="13">
         <v>8</v>
@@ -10395,25 +10395,25 @@
   <sheetData>
     <row r="1" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="E1" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="D1" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E1" s="12" t="s">
+      <c r="F1" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="12" t="s">
         <v>186</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -10424,7 +10424,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D2" s="13">
         <v>16</v>
@@ -10447,7 +10447,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D3" s="13">
         <v>17</v>
@@ -10470,7 +10470,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D4" s="13">
         <v>16</v>
@@ -10493,7 +10493,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D5" s="13">
         <v>18</v>
@@ -10516,7 +10516,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D6" s="13">
         <v>19</v>
@@ -10539,7 +10539,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D7" s="13">
         <v>20</v>
@@ -10562,7 +10562,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D8" s="13">
         <v>3</v>
@@ -10585,7 +10585,7 @@
         <v>15</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D9" s="13">
         <v>21</v>
@@ -10608,7 +10608,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D10" s="13">
         <v>22</v>
@@ -10631,7 +10631,7 @@
         <v>15</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D11" s="13">
         <v>3</v>
@@ -10654,7 +10654,7 @@
         <v>16</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D12" s="13">
         <v>22</v>
@@ -10677,7 +10677,7 @@
         <v>16</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D13" s="13">
         <v>21</v>
@@ -10700,7 +10700,7 @@
         <v>16</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D14" s="13">
         <v>3</v>
@@ -10723,7 +10723,7 @@
         <v>16</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D15" s="13">
         <v>3</v>
@@ -10746,7 +10746,7 @@
         <v>16</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D16" s="13">
         <v>3</v>
@@ -10769,7 +10769,7 @@
         <v>21</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D17" s="13">
         <v>23</v>
@@ -10792,7 +10792,7 @@
         <v>21</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D18" s="13">
         <v>23</v>
@@ -10815,7 +10815,7 @@
         <v>21</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D19" s="17">
         <v>41</v>
@@ -10838,7 +10838,7 @@
         <v>21</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D20" s="13">
         <v>24</v>
@@ -10861,7 +10861,7 @@
         <v>21</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D21" s="13">
         <v>16</v>
@@ -10884,7 +10884,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D22" s="13">
         <v>3</v>
@@ -10907,7 +10907,7 @@
         <v>23</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D23" s="13">
         <v>23</v>
@@ -10930,7 +10930,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D24" s="13">
         <v>3</v>
@@ -10953,7 +10953,7 @@
         <v>23</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D25" s="13">
         <v>22</v>
@@ -10976,7 +10976,7 @@
         <v>27</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D26" s="13">
         <v>3</v>
@@ -10999,7 +10999,7 @@
         <v>27</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D27" s="13">
         <v>3</v>
@@ -11022,7 +11022,7 @@
         <v>28</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D28" s="13">
         <v>3</v>
@@ -11045,7 +11045,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D29" s="13">
         <v>25</v>
@@ -11068,7 +11068,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D30" s="13">
         <v>26</v>
@@ -11091,7 +11091,7 @@
         <v>34</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D31" s="13">
         <v>27</v>
@@ -11114,7 +11114,7 @@
         <v>34</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D32" s="13">
         <v>28</v>
@@ -11137,7 +11137,7 @@
         <v>36</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D33" s="13">
         <v>3</v>

</xml_diff>

<commit_message>
restablecer contraseña, actualizar perfil,bitacora gasto en ConsultaGastos.jsx, contraseña "12345678" para todos los usuarios
</commit_message>
<xml_diff>
--- a/data/datos_reales/xlsx/DatosReales_CICES_Personal.xlsx
+++ b/data/datos_reales/xlsx/DatosReales_CICES_Personal.xlsx
@@ -1,27 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angie\IdeaProjects\cices-system\data\datos_reales\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D27D25A-6132-4F6E-8E01-C82FA1137FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D894FBA2-5228-4EAA-8AD6-E52E855B6033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="USUARIO" sheetId="1" r:id="rId1"/>
     <sheet name="EMPLEADO" sheetId="2" r:id="rId2"/>
-    <sheet name="ROL_USUARIO" sheetId="4" r:id="rId3"/>
-    <sheet name="INVESTIGADOR" sheetId="5" r:id="rId4"/>
+    <sheet name="INVESTIGADOR" sheetId="5" r:id="rId3"/>
+    <sheet name="ROL_USUARIO" sheetId="4" r:id="rId4"/>
     <sheet name="TITULO" sheetId="6" r:id="rId5"/>
     <sheet name="CERTIFICACION" sheetId="7" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId11" roundtripDataChecksum="DFS16W5GeHNxkwd5Blay9s1/ie7Splr6EbD/nyZ3Ff4="/>
     </ext>
@@ -30,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="221">
   <si>
     <t>ID_USUARIO</t>
   </si>
@@ -686,7 +697,13 @@
     <t>Actualización en el manejo de desechos sólidos hospitalarios y técnicas aséptica médico quirúrgica</t>
   </si>
   <si>
-    <t>$2a$10$kWDYd0ioPAF98lxQHAxGaewL3jBNgGqTFwn95532pPwCAKETwTKae</t>
+    <t>prueba1@ucr.ac.cr</t>
+  </si>
+  <si>
+    <t>$2a$10$qWLHzua1Mn5S3cuAYTFuOeVG7FtlA.Q5VmBnxIVIE.hbwRwXebvQ.</t>
+  </si>
+  <si>
+    <t>prueba1</t>
   </si>
 </sst>
 </file>
@@ -697,7 +714,7 @@
     <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -750,6 +767,13 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -768,10 +792,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -808,8 +833,10 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1054,7 +1081,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D2" s="4">
         <v>1</v>
@@ -1068,7 +1095,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D3" s="4">
         <v>1</v>
@@ -1082,7 +1109,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D4" s="4">
         <v>1</v>
@@ -1096,7 +1123,7 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D5" s="4">
         <v>1</v>
@@ -1110,7 +1137,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D6" s="4">
         <v>1</v>
@@ -1124,7 +1151,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D7" s="4">
         <v>1</v>
@@ -1138,7 +1165,7 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D8" s="4">
         <v>1</v>
@@ -1152,7 +1179,7 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D9" s="4">
         <v>1</v>
@@ -1166,7 +1193,7 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D10" s="4">
         <v>1</v>
@@ -1180,7 +1207,7 @@
         <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D11" s="4">
         <v>1</v>
@@ -1194,7 +1221,7 @@
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D12" s="4">
         <v>1</v>
@@ -1208,7 +1235,7 @@
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D13" s="4">
         <v>1</v>
@@ -1222,7 +1249,7 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D14" s="4">
         <v>1</v>
@@ -1236,7 +1263,7 @@
         <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D15" s="4">
         <v>1</v>
@@ -1250,7 +1277,7 @@
         <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D16" s="4">
         <v>1</v>
@@ -1264,7 +1291,7 @@
         <v>19</v>
       </c>
       <c r="C17" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D17" s="4">
         <v>1</v>
@@ -1278,7 +1305,7 @@
         <v>20</v>
       </c>
       <c r="C18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D18" s="4">
         <v>1</v>
@@ -1292,7 +1319,7 @@
         <v>21</v>
       </c>
       <c r="C19" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D19" s="4">
         <v>1</v>
@@ -1306,7 +1333,7 @@
         <v>22</v>
       </c>
       <c r="C20" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D20" s="4">
         <v>1</v>
@@ -1320,7 +1347,7 @@
         <v>23</v>
       </c>
       <c r="C21" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D21" s="4">
         <v>1</v>
@@ -1334,7 +1361,7 @@
         <v>24</v>
       </c>
       <c r="C22" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D22" s="4">
         <v>1</v>
@@ -1348,7 +1375,7 @@
         <v>25</v>
       </c>
       <c r="C23" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D23" s="4">
         <v>1</v>
@@ -1362,7 +1389,7 @@
         <v>26</v>
       </c>
       <c r="C24" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D24" s="4">
         <v>1</v>
@@ -1376,7 +1403,7 @@
         <v>27</v>
       </c>
       <c r="C25" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D25" s="4">
         <v>1</v>
@@ -1390,7 +1417,7 @@
         <v>28</v>
       </c>
       <c r="C26" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D26" s="4">
         <v>1</v>
@@ -1404,7 +1431,7 @@
         <v>29</v>
       </c>
       <c r="C27" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D27" s="4">
         <v>1</v>
@@ -1418,7 +1445,7 @@
         <v>30</v>
       </c>
       <c r="C28" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D28" s="4">
         <v>1</v>
@@ -1432,7 +1459,7 @@
         <v>31</v>
       </c>
       <c r="C29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D29" s="4">
         <v>1</v>
@@ -1446,7 +1473,7 @@
         <v>32</v>
       </c>
       <c r="C30" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D30" s="4">
         <v>1</v>
@@ -1460,7 +1487,7 @@
         <v>33</v>
       </c>
       <c r="C31" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D31" s="4">
         <v>1</v>
@@ -1474,7 +1501,7 @@
         <v>34</v>
       </c>
       <c r="C32" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D32" s="4">
         <v>1</v>
@@ -1488,7 +1515,7 @@
         <v>35</v>
       </c>
       <c r="C33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D33" s="4">
         <v>1</v>
@@ -1502,7 +1529,7 @@
         <v>36</v>
       </c>
       <c r="C34" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D34" s="4">
         <v>1</v>
@@ -1516,7 +1543,7 @@
         <v>37</v>
       </c>
       <c r="C35" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D35" s="4">
         <v>1</v>
@@ -1530,7 +1557,7 @@
         <v>38</v>
       </c>
       <c r="C36" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D36" s="5">
         <v>0</v>
@@ -1544,7 +1571,7 @@
         <v>39</v>
       </c>
       <c r="C37" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D37" s="5">
         <v>0</v>
@@ -1558,7 +1585,7 @@
         <v>40</v>
       </c>
       <c r="C38" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D38" s="5">
         <v>0</v>
@@ -1572,7 +1599,7 @@
         <v>41</v>
       </c>
       <c r="C39" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D39" s="5">
         <v>0</v>
@@ -1586,7 +1613,7 @@
         <v>42</v>
       </c>
       <c r="C40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D40" s="5">
         <v>0</v>
@@ -1600,7 +1627,7 @@
         <v>43</v>
       </c>
       <c r="C41" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D41" s="5">
         <v>0</v>
@@ -1614,7 +1641,7 @@
         <v>44</v>
       </c>
       <c r="C42" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D42" s="4">
         <v>1</v>
@@ -1628,7 +1655,7 @@
         <v>45</v>
       </c>
       <c r="C43" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D43" s="4">
         <v>1</v>
@@ -1642,7 +1669,7 @@
         <v>46</v>
       </c>
       <c r="C44" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D44" s="4">
         <v>1</v>
@@ -1656,7 +1683,7 @@
         <v>47</v>
       </c>
       <c r="C45" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D45" s="4">
         <v>1</v>
@@ -1670,7 +1697,7 @@
         <v>48</v>
       </c>
       <c r="C46" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D46" s="4">
         <v>1</v>
@@ -1684,7 +1711,7 @@
         <v>49</v>
       </c>
       <c r="C47" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D47" s="4">
         <v>1</v>
@@ -1698,7 +1725,7 @@
         <v>50</v>
       </c>
       <c r="C48" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D48" s="4">
         <v>1</v>
@@ -1712,7 +1739,7 @@
         <v>51</v>
       </c>
       <c r="C49" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D49" s="4">
         <v>1</v>
@@ -1726,13 +1753,26 @@
         <v>52</v>
       </c>
       <c r="C50" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D50" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="2">
+        <v>50</v>
+      </c>
+      <c r="B51" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="C51" t="s">
+        <v>219</v>
+      </c>
+      <c r="D51" s="4">
+        <v>1</v>
+      </c>
+    </row>
     <row r="52" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="53" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="54" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -2732,6 +2772,7 @@
     <hyperlink ref="B48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
     <hyperlink ref="B49" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
     <hyperlink ref="B50" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="B51" r:id="rId50" xr:uid="{17F12D92-E12B-412D-846C-C34AB8234558}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -4160,7 +4201,35 @@
       </c>
       <c r="J50" s="2"/>
     </row>
-    <row r="51" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="2">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2">
+        <v>50</v>
+      </c>
+      <c r="C51" t="s">
+        <v>220</v>
+      </c>
+      <c r="D51" s="2">
+        <v>111</v>
+      </c>
+      <c r="E51" s="2">
+        <v>1</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G51" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="H51">
+        <v>111</v>
+      </c>
+      <c r="I51" s="2">
+        <v>5</v>
+      </c>
+    </row>
     <row r="52" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="53" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="54" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -5159,6 +5228,7 @@
     <hyperlink ref="G48" r:id="rId47" xr:uid="{00000000-0004-0000-0100-00002E000000}"/>
     <hyperlink ref="G49" r:id="rId48" xr:uid="{00000000-0004-0000-0100-00002F000000}"/>
     <hyperlink ref="G50" r:id="rId49" xr:uid="{00000000-0004-0000-0100-000030000000}"/>
+    <hyperlink ref="G51" r:id="rId50" xr:uid="{B6A9DDF8-CE27-42E2-B158-6100BBB465BD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -5166,610 +5236,813 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C999"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:E999"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" customWidth="1"/>
-    <col min="3" max="3" width="13.77734375" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="8.109375" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="19.21875" customWidth="1"/>
+    <col min="4" max="4" width="23.77734375" customWidth="1"/>
+    <col min="5" max="5" width="57" customWidth="1"/>
+    <col min="6" max="6" width="25.109375" customWidth="1"/>
+    <col min="7" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="4">
         <v>1</v>
       </c>
       <c r="C2" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D2" s="4">
+        <v>3</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
-        <v>1</v>
+      <c r="B3" s="4">
+        <v>2</v>
       </c>
       <c r="C3" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D3" s="4">
+        <v>3</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
-        <v>2</v>
+      <c r="B4" s="4">
+        <v>3</v>
       </c>
       <c r="C4" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+      <c r="D4" s="4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
-        <v>2</v>
+      <c r="B5" s="4">
+        <v>4</v>
       </c>
       <c r="C5" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="D5" s="4">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="4">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4">
+        <v>38</v>
+      </c>
+      <c r="D6" s="4">
         <v>3</v>
       </c>
-      <c r="C6" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E6" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="2">
-        <v>4</v>
+      <c r="B7" s="4">
+        <v>6</v>
       </c>
       <c r="C7" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="D7" s="4">
+        <v>3</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
-      <c r="B8" s="2">
-        <v>5</v>
+      <c r="B8" s="4">
+        <v>7</v>
       </c>
       <c r="C8" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+      <c r="D8" s="4">
+        <v>3</v>
+      </c>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>8</v>
       </c>
-      <c r="B9" s="2">
-        <v>6</v>
+      <c r="B9" s="4">
+        <v>8</v>
       </c>
       <c r="C9" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="D9" s="4">
+        <v>3</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>9</v>
       </c>
-      <c r="B10" s="2">
-        <v>7</v>
+      <c r="B10" s="4">
+        <v>9</v>
       </c>
       <c r="C10" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+      <c r="D10" s="4">
+        <v>3</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>10</v>
       </c>
-      <c r="B11" s="2">
-        <v>8</v>
+      <c r="B11" s="4">
+        <v>10</v>
       </c>
       <c r="C11" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="D11" s="4">
+        <v>3</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>11</v>
       </c>
-      <c r="B12" s="2">
-        <v>9</v>
+      <c r="B12" s="4">
+        <v>11</v>
       </c>
       <c r="C12" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D12" s="4">
+        <v>3</v>
+      </c>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>12</v>
       </c>
-      <c r="B13" s="2">
-        <v>10</v>
+      <c r="B13" s="4">
+        <v>12</v>
       </c>
       <c r="C13" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="D13" s="4">
+        <v>3</v>
+      </c>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>13</v>
       </c>
-      <c r="B14" s="2">
-        <v>11</v>
+      <c r="B14" s="4">
+        <v>13</v>
       </c>
       <c r="C14" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+      <c r="D14" s="4">
+        <v>3</v>
+      </c>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>14</v>
       </c>
-      <c r="B15" s="2">
-        <v>12</v>
+      <c r="B15" s="4">
+        <v>14</v>
       </c>
       <c r="C15" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D15" s="4">
+        <v>3</v>
+      </c>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>15</v>
       </c>
-      <c r="B16" s="2">
-        <v>13</v>
+      <c r="B16" s="4">
+        <v>15</v>
       </c>
       <c r="C16" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D16" s="4">
+        <v>3</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>16</v>
       </c>
-      <c r="B17" s="2">
-        <v>14</v>
+      <c r="B17" s="4">
+        <v>16</v>
       </c>
       <c r="C17" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D17" s="4">
+        <v>3</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>17</v>
       </c>
-      <c r="B18" s="2">
-        <v>15</v>
+      <c r="B18" s="4">
+        <v>17</v>
       </c>
       <c r="C18" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D18" s="4">
+        <v>3</v>
+      </c>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>18</v>
       </c>
-      <c r="B19" s="2">
-        <v>15</v>
+      <c r="B19" s="4">
+        <v>18</v>
       </c>
       <c r="C19" s="4">
+        <v>36</v>
+      </c>
+      <c r="D19" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>19</v>
       </c>
-      <c r="B20" s="2">
-        <v>16</v>
+      <c r="B20" s="4">
+        <v>19</v>
       </c>
       <c r="C20" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D20" s="4">
+        <v>3</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>20</v>
       </c>
-      <c r="B21" s="2">
-        <v>17</v>
+      <c r="B21" s="4">
+        <v>20</v>
       </c>
       <c r="C21" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D21" s="4">
+        <v>3</v>
+      </c>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>21</v>
       </c>
-      <c r="B22" s="2">
-        <v>18</v>
+      <c r="B22" s="4">
+        <v>21</v>
       </c>
       <c r="C22" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D22" s="4">
+        <v>3</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>22</v>
       </c>
-      <c r="B23" s="2">
-        <v>19</v>
+      <c r="B23" s="4">
+        <v>22</v>
       </c>
       <c r="C23" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D23" s="4">
+        <v>3</v>
+      </c>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>23</v>
       </c>
-      <c r="B24" s="2">
-        <v>20</v>
+      <c r="B24" s="4">
+        <v>23</v>
       </c>
       <c r="C24" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D24" s="4">
+        <v>3</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>24</v>
       </c>
-      <c r="B25" s="2">
-        <v>21</v>
+      <c r="B25" s="4">
+        <v>24</v>
       </c>
       <c r="C25" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D25" s="4">
+        <v>3</v>
+      </c>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>25</v>
       </c>
-      <c r="B26" s="2">
-        <v>22</v>
+      <c r="B26" s="4">
+        <v>25</v>
       </c>
       <c r="C26" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D26" s="4">
+        <v>3</v>
+      </c>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>26</v>
       </c>
-      <c r="B27" s="2">
-        <v>23</v>
+      <c r="B27" s="4">
+        <v>26</v>
       </c>
       <c r="C27" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+      <c r="D27" s="4">
+        <v>3</v>
+      </c>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>27</v>
       </c>
-      <c r="B28" s="2">
-        <v>24</v>
+      <c r="B28" s="4">
+        <v>27</v>
       </c>
       <c r="C28" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D28" s="4">
+        <v>3</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>28</v>
       </c>
-      <c r="B29" s="2">
-        <v>25</v>
+      <c r="B29" s="4">
+        <v>28</v>
       </c>
       <c r="C29" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="D29" s="4">
+        <v>3</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>29</v>
       </c>
-      <c r="B30" s="2">
-        <v>26</v>
+      <c r="B30" s="4">
+        <v>29</v>
       </c>
       <c r="C30" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D30" s="4">
+        <v>3</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>30</v>
       </c>
-      <c r="B31" s="2">
-        <v>27</v>
+      <c r="B31" s="4">
+        <v>30</v>
       </c>
       <c r="C31" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D31" s="4">
+        <v>3</v>
+      </c>
+      <c r="E31" s="4"/>
+    </row>
+    <row r="32" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>31</v>
       </c>
-      <c r="B32" s="2">
-        <v>28</v>
+      <c r="B32" s="4">
+        <v>31</v>
       </c>
       <c r="C32" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D32" s="4">
+        <v>3</v>
+      </c>
+      <c r="E32" s="4"/>
+    </row>
+    <row r="33" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>32</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="4">
+        <v>32</v>
+      </c>
+      <c r="C33" s="4">
         <v>29</v>
       </c>
-      <c r="C33" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D33" s="4">
+        <v>3</v>
+      </c>
+      <c r="E33" s="4"/>
+    </row>
+    <row r="34" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>33</v>
       </c>
-      <c r="B34" s="2">
-        <v>30</v>
+      <c r="B34" s="4">
+        <v>33</v>
       </c>
       <c r="C34" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D34" s="4">
+        <v>3</v>
+      </c>
+      <c r="E34" s="4"/>
+    </row>
+    <row r="35" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
         <v>34</v>
       </c>
-      <c r="B35" s="2">
-        <v>31</v>
+      <c r="B35" s="4">
+        <v>34</v>
       </c>
       <c r="C35" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D35" s="4">
+        <v>3</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>35</v>
       </c>
-      <c r="B36" s="2">
-        <v>32</v>
+      <c r="B36" s="4">
+        <v>35</v>
       </c>
       <c r="C36" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D36" s="4">
+        <v>3</v>
+      </c>
+      <c r="E36" s="4"/>
+    </row>
+    <row r="37" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
         <v>36</v>
       </c>
-      <c r="B37" s="2">
-        <v>33</v>
+      <c r="B37" s="4">
+        <v>36</v>
       </c>
       <c r="C37" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D37" s="4">
+        <v>3</v>
+      </c>
+      <c r="E37" s="4"/>
+    </row>
+    <row r="38" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>37</v>
       </c>
-      <c r="B38" s="2">
-        <v>34</v>
+      <c r="B38" s="4">
+        <v>37</v>
       </c>
       <c r="C38" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D38" s="4">
+        <v>3</v>
+      </c>
+      <c r="E38" s="4"/>
+    </row>
+    <row r="39" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
         <v>38</v>
       </c>
-      <c r="B39" s="2">
-        <v>35</v>
+      <c r="B39" s="4">
+        <v>38</v>
       </c>
       <c r="C39" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D39" s="4">
+        <v>3</v>
+      </c>
+      <c r="E39" s="4"/>
+    </row>
+    <row r="40" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>39</v>
       </c>
-      <c r="B40" s="2">
-        <v>36</v>
+      <c r="B40" s="4">
+        <v>39</v>
       </c>
       <c r="C40" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D40" s="4">
+        <v>3</v>
+      </c>
+      <c r="E40" s="4"/>
+    </row>
+    <row r="41" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
         <v>40</v>
       </c>
-      <c r="B41" s="2">
-        <v>37</v>
+      <c r="B41" s="4">
+        <v>40</v>
       </c>
       <c r="C41" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D41" s="4">
+        <v>3</v>
+      </c>
+      <c r="E41" s="4"/>
+    </row>
+    <row r="42" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>41</v>
       </c>
-      <c r="B42" s="2">
-        <v>38</v>
+      <c r="B42" s="4">
+        <v>41</v>
       </c>
       <c r="C42" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="D42" s="4">
+        <v>3</v>
+      </c>
+      <c r="E42" s="4"/>
+    </row>
+    <row r="43" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
         <v>42</v>
       </c>
-      <c r="B43" s="2">
-        <v>39</v>
+      <c r="B43" s="4">
+        <v>42</v>
       </c>
       <c r="C43" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="D43" s="4">
+        <v>3</v>
+      </c>
+      <c r="E43" s="4"/>
+    </row>
+    <row r="44" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>43</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="4">
+        <v>43</v>
+      </c>
+      <c r="C44" s="4">
         <v>40</v>
       </c>
-      <c r="C44" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D44" s="4">
+        <v>3</v>
+      </c>
+      <c r="E44" s="4"/>
+    </row>
+    <row r="45" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
         <v>44</v>
       </c>
-      <c r="B45" s="2">
-        <v>41</v>
+      <c r="B45" s="4">
+        <v>44</v>
       </c>
       <c r="C45" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D45" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
         <v>45</v>
       </c>
-      <c r="B46" s="2">
-        <v>42</v>
+      <c r="B46" s="4">
+        <v>45</v>
       </c>
       <c r="C46" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D46" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
         <v>46</v>
       </c>
-      <c r="B47" s="2">
-        <v>43</v>
+      <c r="B47" s="4">
+        <v>46</v>
       </c>
       <c r="C47" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D47" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
         <v>47</v>
       </c>
-      <c r="B48" s="2">
-        <v>44</v>
+      <c r="B48" s="4">
+        <v>47</v>
       </c>
       <c r="C48" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D48" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
         <v>48</v>
       </c>
-      <c r="B49" s="2">
-        <v>45</v>
+      <c r="B49" s="4">
+        <v>48</v>
       </c>
       <c r="C49" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D49" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
         <v>49</v>
       </c>
-      <c r="B50" s="2">
-        <v>46</v>
+      <c r="B50" s="4">
+        <v>50</v>
       </c>
       <c r="C50" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="4">
-        <v>50</v>
-      </c>
-      <c r="B51" s="2">
-        <v>47</v>
-      </c>
-      <c r="C51" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="4">
-        <v>51</v>
-      </c>
-      <c r="B52" s="2">
-        <v>48</v>
-      </c>
-      <c r="C52" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="4">
-        <v>52</v>
-      </c>
-      <c r="B53" s="2">
-        <v>49</v>
-      </c>
-      <c r="C53" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+        <v>39</v>
+      </c>
+      <c r="D50" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -6712,800 +6985,620 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E999"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:C999"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.109375" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
-    <col min="3" max="3" width="19.21875" customWidth="1"/>
-    <col min="4" max="4" width="23.77734375" customWidth="1"/>
-    <col min="5" max="5" width="57" customWidth="1"/>
-    <col min="6" max="6" width="25.109375" customWidth="1"/>
-    <col min="7" max="26" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <v>1</v>
       </c>
       <c r="C2" s="4">
-        <v>29</v>
-      </c>
-      <c r="D2" s="4">
-        <v>3</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
         <v>2</v>
       </c>
-      <c r="C3" s="4">
-        <v>29</v>
-      </c>
-      <c r="D3" s="4">
-        <v>3</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="4">
-        <v>3</v>
+      <c r="B4" s="2">
+        <v>2</v>
       </c>
       <c r="C4" s="4">
-        <v>32</v>
-      </c>
-      <c r="D4" s="4">
-        <v>3</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="4">
-        <v>4</v>
+      <c r="B5" s="2">
+        <v>2</v>
       </c>
       <c r="C5" s="4">
-        <v>30</v>
-      </c>
-      <c r="D5" s="4">
-        <v>3</v>
-      </c>
-      <c r="E5" s="4"/>
-    </row>
-    <row r="6" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="4">
-        <v>5</v>
+      <c r="B6" s="2">
+        <v>3</v>
       </c>
       <c r="C6" s="4">
-        <v>38</v>
-      </c>
-      <c r="D6" s="4">
-        <v>3</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
-        <v>6</v>
+      <c r="B7" s="2">
+        <v>4</v>
       </c>
       <c r="C7" s="4">
-        <v>31</v>
-      </c>
-      <c r="D7" s="4">
-        <v>3</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
-      <c r="B8" s="4">
-        <v>7</v>
+      <c r="B8" s="2">
+        <v>5</v>
       </c>
       <c r="C8" s="4">
-        <v>32</v>
-      </c>
-      <c r="D8" s="4">
-        <v>3</v>
-      </c>
-      <c r="E8" s="4"/>
-    </row>
-    <row r="9" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>8</v>
       </c>
-      <c r="B9" s="4">
-        <v>8</v>
+      <c r="B9" s="2">
+        <v>6</v>
       </c>
       <c r="C9" s="4">
-        <v>30</v>
-      </c>
-      <c r="D9" s="4">
-        <v>3</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>9</v>
       </c>
-      <c r="B10" s="4">
-        <v>9</v>
+      <c r="B10" s="2">
+        <v>7</v>
       </c>
       <c r="C10" s="4">
-        <v>33</v>
-      </c>
-      <c r="D10" s="4">
-        <v>3</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>10</v>
       </c>
-      <c r="B11" s="4">
-        <v>10</v>
+      <c r="B11" s="2">
+        <v>8</v>
       </c>
       <c r="C11" s="4">
-        <v>34</v>
-      </c>
-      <c r="D11" s="4">
-        <v>3</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>11</v>
       </c>
-      <c r="B12" s="4">
-        <v>11</v>
+      <c r="B12" s="2">
+        <v>9</v>
       </c>
       <c r="C12" s="4">
-        <v>29</v>
-      </c>
-      <c r="D12" s="4">
-        <v>3</v>
-      </c>
-      <c r="E12" s="4"/>
-    </row>
-    <row r="13" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>12</v>
       </c>
-      <c r="B13" s="4">
-        <v>12</v>
+      <c r="B13" s="2">
+        <v>10</v>
       </c>
       <c r="C13" s="4">
-        <v>31</v>
-      </c>
-      <c r="D13" s="4">
-        <v>3</v>
-      </c>
-      <c r="E13" s="4"/>
-    </row>
-    <row r="14" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>13</v>
       </c>
-      <c r="B14" s="4">
-        <v>13</v>
+      <c r="B14" s="2">
+        <v>11</v>
       </c>
       <c r="C14" s="4">
-        <v>35</v>
-      </c>
-      <c r="D14" s="4">
-        <v>3</v>
-      </c>
-      <c r="E14" s="4"/>
-    </row>
-    <row r="15" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>14</v>
       </c>
-      <c r="B15" s="4">
-        <v>14</v>
+      <c r="B15" s="2">
+        <v>12</v>
       </c>
       <c r="C15" s="4">
-        <v>29</v>
-      </c>
-      <c r="D15" s="4">
-        <v>3</v>
-      </c>
-      <c r="E15" s="4"/>
-    </row>
-    <row r="16" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>15</v>
       </c>
-      <c r="B16" s="4">
-        <v>15</v>
+      <c r="B16" s="2">
+        <v>13</v>
       </c>
       <c r="C16" s="4">
-        <v>39</v>
-      </c>
-      <c r="D16" s="4">
-        <v>3</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>16</v>
       </c>
-      <c r="B17" s="4">
-        <v>16</v>
+      <c r="B17" s="2">
+        <v>14</v>
       </c>
       <c r="C17" s="4">
-        <v>29</v>
-      </c>
-      <c r="D17" s="4">
-        <v>3</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>17</v>
       </c>
-      <c r="B18" s="4">
-        <v>17</v>
+      <c r="B18" s="2">
+        <v>15</v>
       </c>
       <c r="C18" s="4">
-        <v>29</v>
-      </c>
-      <c r="D18" s="4">
-        <v>3</v>
-      </c>
-      <c r="E18" s="4"/>
-    </row>
-    <row r="19" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>18</v>
       </c>
-      <c r="B19" s="4">
-        <v>18</v>
+      <c r="B19" s="2">
+        <v>15</v>
       </c>
       <c r="C19" s="4">
-        <v>36</v>
-      </c>
-      <c r="D19" s="4">
         <v>3</v>
       </c>
-      <c r="E19" s="4"/>
-    </row>
-    <row r="20" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>19</v>
       </c>
-      <c r="B20" s="4">
-        <v>19</v>
+      <c r="B20" s="2">
+        <v>16</v>
       </c>
       <c r="C20" s="4">
-        <v>29</v>
-      </c>
-      <c r="D20" s="4">
-        <v>3</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>20</v>
       </c>
-      <c r="B21" s="4">
-        <v>20</v>
+      <c r="B21" s="2">
+        <v>17</v>
       </c>
       <c r="C21" s="4">
-        <v>29</v>
-      </c>
-      <c r="D21" s="4">
-        <v>3</v>
-      </c>
-      <c r="E21" s="4"/>
-    </row>
-    <row r="22" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>21</v>
       </c>
-      <c r="B22" s="4">
-        <v>21</v>
+      <c r="B22" s="2">
+        <v>18</v>
       </c>
       <c r="C22" s="4">
-        <v>29</v>
-      </c>
-      <c r="D22" s="4">
-        <v>3</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>22</v>
       </c>
-      <c r="B23" s="4">
-        <v>22</v>
+      <c r="B23" s="2">
+        <v>19</v>
       </c>
       <c r="C23" s="4">
-        <v>29</v>
-      </c>
-      <c r="D23" s="4">
-        <v>3</v>
-      </c>
-      <c r="E23" s="4"/>
-    </row>
-    <row r="24" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>23</v>
       </c>
-      <c r="B24" s="4">
-        <v>23</v>
+      <c r="B24" s="2">
+        <v>20</v>
       </c>
       <c r="C24" s="4">
-        <v>29</v>
-      </c>
-      <c r="D24" s="4">
-        <v>3</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>24</v>
       </c>
-      <c r="B25" s="4">
-        <v>24</v>
+      <c r="B25" s="2">
+        <v>21</v>
       </c>
       <c r="C25" s="4">
-        <v>29</v>
-      </c>
-      <c r="D25" s="4">
-        <v>3</v>
-      </c>
-      <c r="E25" s="4"/>
-    </row>
-    <row r="26" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>25</v>
       </c>
-      <c r="B26" s="4">
-        <v>25</v>
+      <c r="B26" s="2">
+        <v>22</v>
       </c>
       <c r="C26" s="4">
-        <v>29</v>
-      </c>
-      <c r="D26" s="4">
-        <v>3</v>
-      </c>
-      <c r="E26" s="4"/>
-    </row>
-    <row r="27" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>26</v>
       </c>
-      <c r="B27" s="4">
-        <v>26</v>
+      <c r="B27" s="2">
+        <v>23</v>
       </c>
       <c r="C27" s="4">
-        <v>37</v>
-      </c>
-      <c r="D27" s="4">
-        <v>3</v>
-      </c>
-      <c r="E27" s="4"/>
-    </row>
-    <row r="28" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>27</v>
       </c>
-      <c r="B28" s="4">
-        <v>27</v>
+      <c r="B28" s="2">
+        <v>24</v>
       </c>
       <c r="C28" s="4">
-        <v>29</v>
-      </c>
-      <c r="D28" s="4">
-        <v>3</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>28</v>
       </c>
-      <c r="B29" s="4">
-        <v>28</v>
+      <c r="B29" s="2">
+        <v>25</v>
       </c>
       <c r="C29" s="4">
-        <v>38</v>
-      </c>
-      <c r="D29" s="4">
-        <v>3</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>29</v>
       </c>
-      <c r="B30" s="4">
-        <v>29</v>
+      <c r="B30" s="2">
+        <v>26</v>
       </c>
       <c r="C30" s="4">
-        <v>29</v>
-      </c>
-      <c r="D30" s="4">
-        <v>3</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>30</v>
       </c>
-      <c r="B31" s="4">
-        <v>30</v>
+      <c r="B31" s="2">
+        <v>27</v>
       </c>
       <c r="C31" s="4">
-        <v>29</v>
-      </c>
-      <c r="D31" s="4">
-        <v>3</v>
-      </c>
-      <c r="E31" s="4"/>
-    </row>
-    <row r="32" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>31</v>
       </c>
-      <c r="B32" s="4">
-        <v>31</v>
+      <c r="B32" s="2">
+        <v>28</v>
       </c>
       <c r="C32" s="4">
-        <v>29</v>
-      </c>
-      <c r="D32" s="4">
-        <v>3</v>
-      </c>
-      <c r="E32" s="4"/>
-    </row>
-    <row r="33" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>32</v>
       </c>
-      <c r="B33" s="4">
-        <v>32</v>
+      <c r="B33" s="2">
+        <v>29</v>
       </c>
       <c r="C33" s="4">
-        <v>29</v>
-      </c>
-      <c r="D33" s="4">
-        <v>3</v>
-      </c>
-      <c r="E33" s="4"/>
-    </row>
-    <row r="34" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>33</v>
       </c>
-      <c r="B34" s="4">
-        <v>33</v>
+      <c r="B34" s="2">
+        <v>30</v>
       </c>
       <c r="C34" s="4">
-        <v>29</v>
-      </c>
-      <c r="D34" s="4">
-        <v>3</v>
-      </c>
-      <c r="E34" s="4"/>
-    </row>
-    <row r="35" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
         <v>34</v>
       </c>
-      <c r="B35" s="4">
-        <v>34</v>
+      <c r="B35" s="2">
+        <v>31</v>
       </c>
       <c r="C35" s="4">
-        <v>29</v>
-      </c>
-      <c r="D35" s="4">
-        <v>3</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>35</v>
       </c>
-      <c r="B36" s="4">
-        <v>35</v>
+      <c r="B36" s="2">
+        <v>32</v>
       </c>
       <c r="C36" s="4">
-        <v>39</v>
-      </c>
-      <c r="D36" s="4">
-        <v>3</v>
-      </c>
-      <c r="E36" s="4"/>
-    </row>
-    <row r="37" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
         <v>36</v>
       </c>
-      <c r="B37" s="4">
-        <v>36</v>
+      <c r="B37" s="2">
+        <v>33</v>
       </c>
       <c r="C37" s="4">
-        <v>39</v>
-      </c>
-      <c r="D37" s="4">
-        <v>3</v>
-      </c>
-      <c r="E37" s="4"/>
-    </row>
-    <row r="38" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>37</v>
       </c>
-      <c r="B38" s="4">
-        <v>37</v>
+      <c r="B38" s="2">
+        <v>34</v>
       </c>
       <c r="C38" s="4">
-        <v>39</v>
-      </c>
-      <c r="D38" s="4">
-        <v>3</v>
-      </c>
-      <c r="E38" s="4"/>
-    </row>
-    <row r="39" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
         <v>38</v>
       </c>
-      <c r="B39" s="4">
-        <v>38</v>
+      <c r="B39" s="2">
+        <v>35</v>
       </c>
       <c r="C39" s="4">
-        <v>39</v>
-      </c>
-      <c r="D39" s="4">
-        <v>3</v>
-      </c>
-      <c r="E39" s="4"/>
-    </row>
-    <row r="40" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>39</v>
       </c>
-      <c r="B40" s="4">
-        <v>39</v>
+      <c r="B40" s="2">
+        <v>36</v>
       </c>
       <c r="C40" s="4">
-        <v>39</v>
-      </c>
-      <c r="D40" s="4">
-        <v>3</v>
-      </c>
-      <c r="E40" s="4"/>
-    </row>
-    <row r="41" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
         <v>40</v>
       </c>
-      <c r="B41" s="4">
-        <v>40</v>
+      <c r="B41" s="2">
+        <v>37</v>
       </c>
       <c r="C41" s="4">
-        <v>39</v>
-      </c>
-      <c r="D41" s="4">
-        <v>3</v>
-      </c>
-      <c r="E41" s="4"/>
-    </row>
-    <row r="42" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>41</v>
       </c>
-      <c r="B42" s="4">
-        <v>41</v>
+      <c r="B42" s="2">
+        <v>38</v>
       </c>
       <c r="C42" s="4">
-        <v>40</v>
-      </c>
-      <c r="D42" s="4">
-        <v>3</v>
-      </c>
-      <c r="E42" s="4"/>
-    </row>
-    <row r="43" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
         <v>42</v>
       </c>
-      <c r="B43" s="4">
-        <v>42</v>
+      <c r="B43" s="2">
+        <v>39</v>
       </c>
       <c r="C43" s="4">
-        <v>40</v>
-      </c>
-      <c r="D43" s="4">
-        <v>3</v>
-      </c>
-      <c r="E43" s="4"/>
-    </row>
-    <row r="44" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>43</v>
       </c>
-      <c r="B44" s="4">
-        <v>43</v>
+      <c r="B44" s="2">
+        <v>40</v>
       </c>
       <c r="C44" s="4">
-        <v>40</v>
-      </c>
-      <c r="D44" s="4">
-        <v>3</v>
-      </c>
-      <c r="E44" s="4"/>
-    </row>
-    <row r="45" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
         <v>44</v>
       </c>
-      <c r="B45" s="4">
-        <v>44</v>
+      <c r="B45" s="2">
+        <v>41</v>
       </c>
       <c r="C45" s="4">
-        <v>29</v>
-      </c>
-      <c r="D45" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
         <v>45</v>
       </c>
-      <c r="B46" s="4">
-        <v>45</v>
+      <c r="B46" s="2">
+        <v>42</v>
       </c>
       <c r="C46" s="4">
-        <v>29</v>
-      </c>
-      <c r="D46" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
         <v>46</v>
       </c>
-      <c r="B47" s="4">
-        <v>46</v>
+      <c r="B47" s="2">
+        <v>43</v>
       </c>
       <c r="C47" s="4">
-        <v>29</v>
-      </c>
-      <c r="D47" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
         <v>47</v>
       </c>
-      <c r="B48" s="4">
-        <v>47</v>
+      <c r="B48" s="2">
+        <v>44</v>
       </c>
       <c r="C48" s="4">
-        <v>29</v>
-      </c>
-      <c r="D48" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
         <v>48</v>
       </c>
-      <c r="B49" s="4">
+      <c r="B49" s="2">
+        <v>45</v>
+      </c>
+      <c r="C49" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="4">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2">
+        <v>46</v>
+      </c>
+      <c r="C50" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="4">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2">
+        <v>47</v>
+      </c>
+      <c r="C51" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="4">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2">
         <v>48</v>
       </c>
-      <c r="C49" s="4">
-        <v>29</v>
-      </c>
-      <c r="D49" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="C52" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="4">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2">
+        <v>49</v>
+      </c>
+      <c r="C53" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="4">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2">
+        <v>50</v>
+      </c>
+      <c r="C54" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -10435,9 +10528,7 @@
       <c r="F2" s="16">
         <v>47635</v>
       </c>
-      <c r="G2" s="13">
-        <v>12</v>
-      </c>
+      <c r="G2" s="13"/>
     </row>
     <row r="3" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="13">
@@ -10458,9 +10549,7 @@
       <c r="F3" s="16">
         <v>47635</v>
       </c>
-      <c r="G3" s="13">
-        <v>12</v>
-      </c>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="13">
@@ -10481,9 +10570,7 @@
       <c r="F4" s="16">
         <v>47635</v>
       </c>
-      <c r="G4" s="13">
-        <v>12</v>
-      </c>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
@@ -10504,9 +10591,7 @@
       <c r="F5" s="16">
         <v>41275</v>
       </c>
-      <c r="G5" s="13">
-        <v>14</v>
-      </c>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13">
@@ -10527,9 +10612,7 @@
       <c r="F6" s="16">
         <v>40909</v>
       </c>
-      <c r="G6" s="13">
-        <v>14</v>
-      </c>
+      <c r="G6" s="13"/>
     </row>
     <row r="7" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="13">
@@ -10550,9 +10633,7 @@
       <c r="F7" s="16">
         <v>40544</v>
       </c>
-      <c r="G7" s="13">
-        <v>14</v>
-      </c>
+      <c r="G7" s="13"/>
     </row>
     <row r="8" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
@@ -10573,9 +10654,7 @@
       <c r="F8" s="16">
         <v>37257</v>
       </c>
-      <c r="G8" s="13">
-        <v>14</v>
-      </c>
+      <c r="G8" s="13"/>
     </row>
     <row r="9" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
@@ -10596,9 +10675,7 @@
       <c r="F9" s="16">
         <v>44927</v>
       </c>
-      <c r="G9" s="13">
-        <v>12</v>
-      </c>
+      <c r="G9" s="13"/>
     </row>
     <row r="10" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
@@ -10619,9 +10696,7 @@
       <c r="F10" s="16">
         <v>44927</v>
       </c>
-      <c r="G10" s="13">
-        <v>12</v>
-      </c>
+      <c r="G10" s="13"/>
     </row>
     <row r="11" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
@@ -10642,9 +10717,7 @@
       <c r="F11" s="16">
         <v>44197</v>
       </c>
-      <c r="G11" s="13">
-        <v>12</v>
-      </c>
+      <c r="G11" s="13"/>
     </row>
     <row r="12" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
@@ -10665,9 +10738,7 @@
       <c r="F12" s="16">
         <v>42736</v>
       </c>
-      <c r="G12" s="13">
-        <v>12</v>
-      </c>
+      <c r="G12" s="13"/>
     </row>
     <row r="13" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
@@ -10688,9 +10759,7 @@
       <c r="F13" s="16">
         <v>42736</v>
       </c>
-      <c r="G13" s="13">
-        <v>12</v>
-      </c>
+      <c r="G13" s="13"/>
     </row>
     <row r="14" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13">
@@ -10711,9 +10780,7 @@
       <c r="F14" s="16">
         <v>43831</v>
       </c>
-      <c r="G14" s="13">
-        <v>12</v>
-      </c>
+      <c r="G14" s="13"/>
     </row>
     <row r="15" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13">
@@ -10734,9 +10801,7 @@
       <c r="F15" s="16">
         <v>43466</v>
       </c>
-      <c r="G15" s="13">
-        <v>12</v>
-      </c>
+      <c r="G15" s="13"/>
     </row>
     <row r="16" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13">
@@ -10757,9 +10822,7 @@
       <c r="F16" s="16">
         <v>42370</v>
       </c>
-      <c r="G16" s="13">
-        <v>12</v>
-      </c>
+      <c r="G16" s="13"/>
     </row>
     <row r="17" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="13">
@@ -10780,9 +10843,7 @@
       <c r="F17" s="16">
         <v>47635</v>
       </c>
-      <c r="G17" s="13">
-        <v>12</v>
-      </c>
+      <c r="G17" s="13"/>
     </row>
     <row r="18" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="13">
@@ -10803,9 +10864,7 @@
       <c r="F18" s="16">
         <v>47635</v>
       </c>
-      <c r="G18" s="13">
-        <v>12</v>
-      </c>
+      <c r="G18" s="13"/>
     </row>
     <row r="19" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="13">
@@ -10826,9 +10885,7 @@
       <c r="F19" s="14">
         <v>47635</v>
       </c>
-      <c r="G19" s="13">
-        <v>12</v>
-      </c>
+      <c r="G19" s="13"/>
     </row>
     <row r="20" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="13">
@@ -10849,9 +10906,7 @@
       <c r="F20" s="16">
         <v>47635</v>
       </c>
-      <c r="G20" s="13">
-        <v>12</v>
-      </c>
+      <c r="G20" s="13"/>
     </row>
     <row r="21" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="13">
@@ -10872,9 +10927,7 @@
       <c r="F21" s="16">
         <v>46631</v>
       </c>
-      <c r="G21" s="13">
-        <v>12</v>
-      </c>
+      <c r="G21" s="13"/>
     </row>
     <row r="22" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="13">
@@ -10895,9 +10948,7 @@
       <c r="F22" s="16">
         <v>39814</v>
       </c>
-      <c r="G22" s="13">
-        <v>14</v>
-      </c>
+      <c r="G22" s="13"/>
     </row>
     <row r="23" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="13">
@@ -10918,9 +10969,7 @@
       <c r="F23" s="16">
         <v>42370</v>
       </c>
-      <c r="G23" s="13">
-        <v>14</v>
-      </c>
+      <c r="G23" s="13"/>
     </row>
     <row r="24" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="13">
@@ -10941,9 +10990,7 @@
       <c r="F24" s="16">
         <v>43101</v>
       </c>
-      <c r="G24" s="13">
-        <v>14</v>
-      </c>
+      <c r="G24" s="13"/>
     </row>
     <row r="25" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="13">
@@ -10964,9 +11011,7 @@
       <c r="F25" s="16">
         <v>45658</v>
       </c>
-      <c r="G25" s="17">
-        <v>14</v>
-      </c>
+      <c r="G25" s="17"/>
     </row>
     <row r="26" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="13">
@@ -10987,9 +11032,7 @@
       <c r="F26" s="16">
         <v>43101</v>
       </c>
-      <c r="G26" s="13">
-        <v>14</v>
-      </c>
+      <c r="G26" s="13"/>
     </row>
     <row r="27" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="13">
@@ -11010,9 +11053,7 @@
       <c r="F27" s="16">
         <v>43831</v>
       </c>
-      <c r="G27" s="13">
-        <v>14</v>
-      </c>
+      <c r="G27" s="13"/>
     </row>
     <row r="28" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="13">
@@ -11033,9 +11074,7 @@
       <c r="F28" s="16">
         <v>42005</v>
       </c>
-      <c r="G28" s="13">
-        <v>14</v>
-      </c>
+      <c r="G28" s="13"/>
     </row>
     <row r="29" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="13">
@@ -11056,9 +11095,7 @@
       <c r="F29" s="16">
         <v>44197</v>
       </c>
-      <c r="G29" s="13">
-        <v>14</v>
-      </c>
+      <c r="G29" s="13"/>
     </row>
     <row r="30" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="13">
@@ -11079,9 +11116,7 @@
       <c r="F30" s="16">
         <v>40179</v>
       </c>
-      <c r="G30" s="13">
-        <v>14</v>
-      </c>
+      <c r="G30" s="13"/>
     </row>
     <row r="31" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="13">
@@ -11102,9 +11137,7 @@
       <c r="F31" s="16">
         <v>47635</v>
       </c>
-      <c r="G31" s="13">
-        <v>12</v>
-      </c>
+      <c r="G31" s="13"/>
     </row>
     <row r="32" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="13">
@@ -11125,9 +11158,7 @@
       <c r="F32" s="16">
         <v>47635</v>
       </c>
-      <c r="G32" s="13">
-        <v>12</v>
-      </c>
+      <c r="G32" s="13"/>
     </row>
     <row r="33" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="13">
@@ -11148,9 +11179,7 @@
       <c r="F33" s="16">
         <v>47635</v>
       </c>
-      <c r="G33" s="13">
-        <v>12</v>
-      </c>
+      <c r="G33" s="13"/>
     </row>
     <row r="34" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>

</xml_diff>